<commit_message>
Mark sign-in persistence fix (#54) as user-confirmed resolved
Removed from context.md's backlog, added a confirmation note to History,
and flipped ticket #54 to Done in the tracker.
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -3369,9 +3369,9 @@
           <t>Guarded the auto-reload to defer while the URL still looks like an in-progress auth redirect (8s backstop); added an always-on console diagnostic to confirm a recurrence for certain.</t>
         </is>
       </c>
-      <c r="H58" s="12" t="inlineStr">
-        <is>
-          <t>Needs Testing</t>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I58" s="8" t="inlineStr">
@@ -3381,7 +3381,7 @@
       </c>
       <c r="J58" s="8" t="inlineStr">
         <is>
-          <t>Root cause not fully confirmed -- watch for a recurrence and check the console diagnostic if it happens again.</t>
+          <t>Root cause not fully confirmed -- watch for a recurrence and check the console diagnostic if it happens again. User-confirmed resolved 2026-07-23.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: mark tickets #56, #57, #58 as Done
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -3461,17 +3461,17 @@
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>Not yet investigated.</t>
+          <t>Root cause found: .nav-btn had exactly two fixed sizes (a mobile-and-below size and a 768px+ size) with nothing tuned for a real phone width in between -- an iPhone never reaches the 768px breakpoint, so it always rendered at the larger-than-intended "mobile" size.</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>Not started.</t>
-        </is>
-      </c>
-      <c r="H60" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Replaced the two fixed sizes with clamp()-based fluid scaling for font-size/padding/min-width: max end reproduces the existing 768px+ look unchanged, min end is a legible ~12pt floor, scaling continuously with viewport width in between.</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I60" s="8" t="inlineStr">
@@ -3481,7 +3481,7 @@
       </c>
       <c r="J60" s="8" t="inlineStr">
         <is>
-          <t>Should scale with screen size -- max size is the current fixed size, min size is roughly 12pt-legible.</t>
+          <t>Verified via Playwright: computed font-size/min-width hit exactly 16px/64px at 360px width and 19px/100px at 1024px+, matching the old fixed values at both reference points.</t>
         </is>
       </c>
     </row>
@@ -3511,17 +3511,17 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Not yet investigated.</t>
+          <t>Present's top bar (#presentTop) used overflow-x:auto as its only overflow fallback, with nothing pinned outside it -- on a real phone, brand+timer+sermon-info could still overflow even after existing shrinking, pushing the font-size/dark-mode buttons (the last children) past the right edge, reachable only by an undiscovered scroll.</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>Not started.</t>
-        </is>
-      </c>
-      <c r="H61" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Wrapped brand+timer+sermon-info in a new inner .present-top-scroll wrapper (scrolls independently if needed); .top-actions (font size, dark mode) now sits pinned outside it, always fully visible -- the same pattern Practice's Finish button already used.</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Verified at a real iPhone-class viewport (393px): both buttons measured fully within bounds and confirmed actually clickable with zero scroll, including a worst-case long-title stress test.</t>
         </is>
       </c>
     </row>
@@ -3561,17 +3561,17 @@
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>Not yet investigated.</t>
+          <t>Practice's top bar had already pinned Finish outside its scroller (a prior fix), but Notes/Takes/dark-toggle were still living inside it -- the identical failure mode Finish was pulled out to avoid, just not yet applied to its siblings.</t>
         </is>
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>Not started.</t>
-        </is>
-      </c>
-      <c r="H62" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Moved .top-actions (Notes, Takes, dark-toggle) out to sit pinned between the scroller and Finish, so every control that must never be scrolled out of reach is now consistently pinned, leaving only the informational timer/sermon-name content inside the scroller.</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I62" s="8" t="inlineStr">
@@ -3581,7 +3581,7 @@
       </c>
       <c r="J62" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Verified at a real iPhone-class viewport: Notes/Takes/dark-toggle/Finish all measured fully within bounds, Notes confirmed actually clickable with zero scroll, including a worst-case long-title stress test.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct tracker: #56-58 back to Needs Testing, add real commit timestamps
Real-device-reported bugs default to Needs Testing when fixed (not Done)
until the user confirms on actual hardware -- #56-58 were only verified
in a simulated Playwright viewport. Also backfills exact Date/Time (UTC)
from real git commit timestamps for the current session's tickets
(#43-59), and documents both policies on the Legend tab.
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -161,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -219,6 +219,12 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -615,7 +621,7 @@
     <col width="34" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -676,7 +682,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Date / Time (UTC)</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -2824,9 +2830,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="I47" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
+      <c r="I47" s="22" t="inlineStr">
+        <is>
+          <t>2026-07-22 00:46</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
@@ -2874,9 +2880,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="I48" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
+      <c r="I48" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-22 00:46</t>
         </is>
       </c>
       <c r="J48" s="8" t="inlineStr">
@@ -2924,9 +2930,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="I49" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
+      <c r="I49" s="22" t="inlineStr">
+        <is>
+          <t>2026-07-22 00:46</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr">
@@ -2974,9 +2980,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="I50" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
+      <c r="I50" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-22 00:53</t>
         </is>
       </c>
       <c r="J50" s="8" t="inlineStr">
@@ -3024,9 +3030,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="I51" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
+      <c r="I51" s="22" t="inlineStr">
+        <is>
+          <t>2026-07-22 01:06</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
@@ -3074,9 +3080,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="I52" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
+      <c r="I52" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-22 01:06</t>
         </is>
       </c>
       <c r="J52" s="8" t="inlineStr">
@@ -3124,9 +3130,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="I53" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
+      <c r="I53" s="22" t="inlineStr">
+        <is>
+          <t>2026-07-22 02:01</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
@@ -3174,9 +3180,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="I54" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
+      <c r="I54" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-22 02:04</t>
         </is>
       </c>
       <c r="J54" s="8" t="inlineStr">
@@ -3224,9 +3230,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="I55" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
+      <c r="I55" s="22" t="inlineStr">
+        <is>
+          <t>2026-07-22 01:58</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
@@ -3374,9 +3380,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="I58" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
+      <c r="I58" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-22 01:53</t>
         </is>
       </c>
       <c r="J58" s="8" t="inlineStr">
@@ -3424,9 +3430,9 @@
           <t>Needs Testing</t>
         </is>
       </c>
-      <c r="I59" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
+      <c r="I59" s="22" t="inlineStr">
+        <is>
+          <t>2026-07-22 01:49</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
@@ -3469,19 +3475,19 @@
           <t>Replaced the two fixed sizes with clamp()-based fluid scaling for font-size/padding/min-width: max end reproduces the existing 768px+ look unchanged, min end is a legible ~12pt floor, scaling continuously with viewport width in between.</t>
         </is>
       </c>
-      <c r="H60" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="I60" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
+      <c r="H60" s="12" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
+        </is>
+      </c>
+      <c r="I60" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:19</t>
         </is>
       </c>
       <c r="J60" s="8" t="inlineStr">
         <is>
-          <t>Verified via Playwright: computed font-size/min-width hit exactly 16px/64px at 360px width and 19px/100px at 1024px+, matching the old fixed values at both reference points.</t>
+          <t>Verified via Playwright: computed font-size/min-width hit exactly 16px/64px at 360px width and 19px/100px at 1024px+, matching the old fixed values at both reference points. Status corrected from Done to Needs Testing -- verified only in a simulated Playwright viewport, not the actual iPhone 17 Pro. Going forward, any fix for a real-device-reported bug defaults to Needs Testing until you confirm it on the actual hardware, rather than Done on my own testing alone.</t>
         </is>
       </c>
     </row>
@@ -3519,19 +3525,19 @@
           <t>Wrapped brand+timer+sermon-info in a new inner .present-top-scroll wrapper (scrolls independently if needed); .top-actions (font size, dark mode) now sits pinned outside it, always fully visible -- the same pattern Practice's Finish button already used.</t>
         </is>
       </c>
-      <c r="H61" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="I61" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
+      <c r="H61" s="12" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
+        </is>
+      </c>
+      <c r="I61" s="22" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:19</t>
         </is>
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>Verified at a real iPhone-class viewport (393px): both buttons measured fully within bounds and confirmed actually clickable with zero scroll, including a worst-case long-title stress test.</t>
+          <t>Verified at a real iPhone-class viewport (393px): both buttons measured fully within bounds and confirmed actually clickable with zero scroll, including a worst-case long-title stress test. Status corrected from Done to Needs Testing -- verified only in a simulated Playwright viewport, not the actual iPhone 17 Pro. Going forward, any fix for a real-device-reported bug defaults to Needs Testing until you confirm it on the actual hardware, rather than Done on my own testing alone.</t>
         </is>
       </c>
     </row>
@@ -3569,19 +3575,19 @@
           <t>Moved .top-actions (Notes, Takes, dark-toggle) out to sit pinned between the scroller and Finish, so every control that must never be scrolled out of reach is now consistently pinned, leaving only the informational timer/sermon-name content inside the scroller.</t>
         </is>
       </c>
-      <c r="H62" s="6" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="I62" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
+      <c r="H62" s="12" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
+        </is>
+      </c>
+      <c r="I62" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-22 12:19</t>
         </is>
       </c>
       <c r="J62" s="8" t="inlineStr">
         <is>
-          <t>Verified at a real iPhone-class viewport: Notes/Takes/dark-toggle/Finish all measured fully within bounds, Notes confirmed actually clickable with zero scroll, including a worst-case long-title stress test.</t>
+          <t>Verified at a real iPhone-class viewport: Notes/Takes/dark-toggle/Finish all measured fully within bounds, Notes confirmed actually clickable with zero scroll, including a worst-case long-title stress test. Status corrected from Done to Needs Testing -- verified only in a simulated Playwright viewport, not the actual iPhone 17 Pro. Going forward, any fix for a real-device-reported bug defaults to Needs Testing until you confirm it on the actual hardware, rather than Done on my own testing alone.</t>
         </is>
       </c>
     </row>
@@ -3624,9 +3630,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="I63" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
+      <c r="I63" s="22" t="inlineStr">
+        <is>
+          <t>2026-07-22 11:53</t>
         </is>
       </c>
       <c r="J63" s="5" t="inlineStr">
@@ -3653,7 +3659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3760,12 +3766,28 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>•  Date/Time (UTC) reflects the actual commit timestamp for each fix where one exists (from git log), not a guess -- so it may not match your local timezone. Earlier tickets (#1-42) are left as date-only since many bundle several tickets into one commit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>•  A real-device-reported bug (e.g. flagged on a specific phone) defaults to Needs Testing when fixed, not Done -- verifying in this environment's simulated browser viewport is not the same as confirming on the actual hardware. It only flips to Done once you confirm it.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A1:B1"/>
     <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add ticket #60 to tracker: sync duplicate detection
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J63" headerRowCount="1">
-  <autoFilter ref="A4:J63"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J64" headerRowCount="1">
+  <autoFilter ref="A4:J64"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -314,7 +314,7 @@
     <tableColumn id="6" name="Root Cause / Bug"/>
     <tableColumn id="7" name="Fix / Resolution"/>
     <tableColumn id="8" name="Status"/>
-    <tableColumn id="9" name="Date"/>
+    <tableColumn id="9" name="Date / Time (UTC)"/>
     <tableColumn id="10" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J63"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3638,6 +3638,56 @@
       <c r="J63" s="5" t="inlineStr">
         <is>
           <t>Found and fixed live during the user's item-by-item review of #55.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="90" customHeight="1">
+      <c r="A64" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Sync</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Sync duplicate detection: fuzzy title match + forced resolve popup</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>User reported "sync just keeps making duplicates" while validating #55, and correctly suspected the real gap was cross-device consistency, not either existing fix.</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>Neither #55 (identical content under the *same* id) nor #59 (one id's RLS collision) was ever going to catch two genuinely *different* ids a human recognizes as the same sermon -- e.g. each device independently reassigning its own fresh id after a collision. Ordinary id-based sync correctly treats them as unrelated and pulls both to every device forever.</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>Fuzzy title-similarity detection (Levenshtein ratio, excluding differing trailing sequence numbers so series parts like "Pt 1"/"Pt 2" are never flagged) triggers a centered forced modal on navigating to Library (never during Present/Practice) with exact timestamps shown, offering Keep This One / Keep Both. "Keep Both" renames both titles with a distinguishing timestamp suffix instead of a new synced field -- the rename itself propagates through the existing sermons sync path with zero schema change, and doubles as the "already reviewed" signal.</t>
+        </is>
+      </c>
+      <c r="H64" s="12" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>New capability, not a reopen of #55/#59 (see those tickets' Notes). Verified in this environment including a real cross-device propagation simulation, but not yet confirmed by the user on real devices/data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ticket #61 to tracker: Library/Plan filters-tray redesign
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J64" headerRowCount="1">
-  <autoFilter ref="A4:J64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J65" headerRowCount="1">
+  <autoFilter ref="A4:J65"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3688,6 +3688,56 @@
       <c r="J64" s="5" t="inlineStr">
         <is>
           <t>New capability, not a reopen of #55/#59 (see those tickets' Notes). Verified in this environment including a real cross-device propagation simulation, but not yet confirmed by the user on real devices/data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="90" customHeight="1">
+      <c r="A65" s="7" t="n">
+        <v>61</v>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>Library/Plan</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Redesign Library/Plan filtering as multi-select slicer trays</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>User loaded a large bulk test dataset (10 series x 5 sermons) to stress-test decade-scale volume, then asked to try a new filtering strategy: a "Filters" button opening a collapsible left-side tray with slicers (series, year, month, etc.) instead of the existing single-select dropdown/search-bar UI, for both Library and Plan.</t>
+        </is>
+      </c>
+      <c r="F65" s="8" t="inlineStr">
+        <is>
+          <t>Library's old single-select year/series dropdown and Plan's title-search-with-jump both only let a user narrow by one value at a time and don't scale well to browsing years of accumulated sermons/series -- the user wanted to test whether a multi-select slicer-tray pattern works better at that scale.</t>
+        </is>
+      </c>
+      <c r="G65" s="8" t="inlineStr">
+        <is>
+          <t>New left-side drawer modal (`.modal-overlay.drawer-left`) shared in shape by both views, each with independent Set-based multi-select Series/Year/Month checkbox slicers plus a Sermon-title text search and a Clear All Filters button; a badge on the Filters button shows the active-filter count. Built on the user's own explicit answers to 3 design questions: multi-select (not single-select), Sermon slicer is text search (not a checkbox list), and Plan filters narrow the calendar in place with no auto-jump to a month that has matches.</t>
+        </is>
+      </c>
+      <c r="H65" s="12" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
+        </is>
+      </c>
+      <c r="I65" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J65" s="8" t="inlineStr">
+        <is>
+          <t>This is a UX strategy the user explicitly wants to try firsthand against the bulk test dataset already loaded, not just a hardware-confirmation gap -- verified functionally correct in this environment (filter combination logic, badge count, no-auto-jump behavior, full regression suite), but left as Needs Testing pending the user's own hands-on read of whether the new pattern actually works better.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: #61 confirmed Done, add tickets #62-64
User confirmed the filters-tray redesign (#61) works great. Adds
tickets for the manuscript print margin rework (#62), the pinned
Clear All Filters + Plan legend jump/cycle (#63), and the print
self-invocation fix (#64).
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J65" headerRowCount="1">
-  <autoFilter ref="A4:J65"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J68" headerRowCount="1">
+  <autoFilter ref="A4:J68"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3725,19 +3725,169 @@
           <t>New left-side drawer modal (`.modal-overlay.drawer-left`) shared in shape by both views, each with independent Set-based multi-select Series/Year/Month checkbox slicers plus a Sermon-title text search and a Clear All Filters button; a badge on the Filters button shows the active-filter count. Built on the user's own explicit answers to 3 design questions: multi-select (not single-select), Sermon slicer is text search (not a checkbox list), and Plan filters narrow the calendar in place with no auto-jump to a month that has matches.</t>
         </is>
       </c>
-      <c r="H65" s="12" t="inlineStr">
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I65" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J65" s="8" t="inlineStr">
+        <is>
+          <t>This is a UX strategy the user explicitly wants to try firsthand against the bulk test dataset already loaded, not just a hardware-confirmation gap -- verified functionally correct in this environment (filter combination logic, badge count, no-auto-jump behavior, full regression suite), but left as Needs Testing pending the user's own hands-on read of whether the new pattern actually works better. Confirmed by the user: "The filter function works great."</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="100" customHeight="1">
+      <c r="A66" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Prepare/Export</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Improve manuscript print/PDF export margins and default formatting</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>User: "right now it formats like a web page but I want the print settings to closer match a Word doc, improve the margins and default formats."</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>The generated manuscript document had no @page rule at all -- print margins were whatever each browser's own default happened to be -- and used pixel-based font sizes and a narrow centered web-column layout instead of a document layout.</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>Added an explicit `@page{ size:letter; margin:1in }` rule (Word's own default page margin), switched typography to point-based sizing, and gave the pre-print screen view an actual Letter-size page-card look (white page on a gray canvas) instead of a web column. Added orphan/widow and break-avoid hints for section headers and illustration blocks.</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>Superseded in practice, not in intent, by #64 -- this pass fixed the document's own look correctly (confirmed by the user), but the *print dialog itself* showing worse margins than the preview was a separate bug in how print() was being triggered, fixed as its own ticket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="100" customHeight="1">
+      <c r="A67" s="7" t="n">
+        <v>63</v>
+      </c>
+      <c r="B67" s="8" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>Library/Plan</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Pin Clear All Filters to top of trays + Plan legend jump/cycle</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>User, after confirming #61's filter trays work great: "Let's move the clear all filters button towards the top so the user knows it's there right off the bat. Also for plan, let's build in functionality where if the user taps or clicks on a series from the legend below it moves the calendar to the nearest entry from that series, subsequent clicks move to the next entry cycling through."</t>
+        </is>
+      </c>
+      <c r="F67" s="8" t="inlineStr">
+        <is>
+          <t>Clear All Filters sat at the bottom of the scrollable slicer list in both trays, easy to miss on first use. Plan's legend was purely informational (color-dot + series name) with no interaction, even though quickly stepping through one series' entries in date order is a natural companion action to the filters tray's own narrowing.</t>
+        </is>
+      </c>
+      <c r="G67" s="8" t="inlineStr">
+        <is>
+          <t>Moved Clear All Filters to a new `.filter-clear-row`, a sibling of `.scroll` pinned directly under the tray header in both Library's and Plan's trays. Made Plan's legend items clickable: first tap jumps to the series' nearest entry (by date-distance from the currently displayed month); subsequent taps on the same series cycle forward chronologically and wrap around; a per-series cursor persists across clicks and respects active filters; the landed-on day gets a brief gold flash highlight.</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I67" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J67" s="8" t="inlineStr">
+        <is>
+          <t>Pure desktop UI logic (not device-touch-specific), verified with Playwright: nearest-entry jump in either time direction, forward cycling with wraparound, independent per-series cursors, and the pinned button's position -- all confirmed working as specified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="100" customHeight="1">
+      <c r="A68" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Prepare/Export</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Fix manuscript print margins: self-invoke print instead of cross-window call</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>User tested #62 on a real Windows machine: the manuscript popup itself rendered correctly, but the actual print dialog that opened (a system-level flyout for a third-party PDF print driver, no live page-preview thumbnail) showed worse margins than the preview.</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>`exportManuscript()` called `.print()` on the popup window *from the opener's own script* (`w.print()` inside a `setTimeout`), a known source of a print job losing track of which document's `@page` rule applies, and of some browsers falling back to a bare system print dialog instead of their normal in-page print-preview pipeline that actually reads `@page`.</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>Moved the print trigger into the generated document itself: an inline script inside the manuscript's own HTML calls `window.print()` from a `load` listener, matching what a manual Ctrl+P on that tab would do. Had to escape the injected script's own closing tag (`&lt;\/script&gt;`) since the literal `&lt;/script&gt;` inside the outer app's single big inline `&lt;script&gt;` block (built via a JS template literal) was read by the HTML parser as ending *that* script early, throwing `Unexpected end of input` -- the same trap already solved once for the RevenueCat plugin's conditional `document.write`.</t>
+        </is>
+      </c>
+      <c r="H68" s="12" t="inlineStr">
         <is>
           <t>Needs Testing</t>
         </is>
       </c>
-      <c r="I65" s="8" t="inlineStr">
+      <c r="I68" s="5" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="J65" s="8" t="inlineStr">
-        <is>
-          <t>This is a UX strategy the user explicitly wants to try firsthand against the bulk test dataset already loaded, not just a hardware-confirmation gap -- verified functionally correct in this environment (filter combination logic, badge count, no-auto-jump behavior, full regression suite), but left as Needs Testing pending the user's own hands-on read of whether the new pattern actually works better.</t>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>The real-world margin behavior can only be confirmed by the user re-printing on the same Windows machine/driver that showed the original bug -- verified in this environment that the popup's own script now correctly self-invokes print (via a stubbed window.print(), since headless Chromium has no display to dismiss a real print dialog) and that the rest of the app still parses/runs correctly.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add tickets #65-66: No Series bucket/series-grouped Library, PP tags
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J68" headerRowCount="1">
-  <autoFilter ref="A4:J68"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J70" headerRowCount="1">
+  <autoFilter ref="A4:J70"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3888,6 +3888,106 @@
       <c r="J68" s="5" t="inlineStr">
         <is>
           <t>The real-world margin behavior can only be confirmed by the user re-printing on the same Windows machine/driver that showed the original bug -- verified in this environment that the popup's own script now correctly self-invokes print (via a stubbed window.print(), since headless Chromium has no display to dismiss a real print dialog) and that the rest of the app still parses/runs correctly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="100" customHeight="1">
+      <c r="A69" s="7" t="n">
+        <v>65</v>
+      </c>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Add "No Series" catch-all + regroup Library into collapsible per-series sections</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>User: "let's add a new default series for all messages not associated with a series so they can be located easily as well... What do you think about switching the library view to be by series instead of sermon. Each one starts collapsed and can be expanded to show the indwelling sermons."</t>
+        </is>
+      </c>
+      <c r="F69" s="8" t="inlineStr">
+        <is>
+          <t>Sermons without a series had no way to show up in the Series filter/slicer at all (filtered out as falsy), and the flat sermon-card list got harder to scan as the library grows across years/series.</t>
+        </is>
+      </c>
+      <c r="G69" s="8" t="inlineStr">
+        <is>
+          <t>Any series-less sermon is folded into a fixed "No Series" label everywhere series is used for grouping/filtering/matching (computed at render time, never written back onto the sermon record). Library is now one collapsible section per series -- starts collapsed, "No Series" always sorted last. The existing Recent/By Date sort toggle now orders both the groups themselves and the sermons within each group; any active filter/search force-expands only the groups that still have a match.</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I69" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J69" s="8" t="inlineStr">
+        <is>
+          <t>Verified with Playwright: collapsed-by-default, correct group/sermon ordering under both sort modes, "No Series" present as a real filterable option in both Library's and Plan's Series slicers, and filtering force-expands only the matching group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="100" customHeight="1">
+      <c r="A70" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Prepare/Export</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Add per-item "Slide" toggle to control ProPresenter export inclusion</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>User: "let's add a way to determine on the prepare page which items should be included in the pro presenter export. a tag or something like that."</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>The ProPresenter export was hard-coded to scripture + illustration items only, with no way to include a key block/application point or exclude a scripture reference that's in the manuscript but not meant to be projected.</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>Added a small "Slide" toggle pill to every item row (`it.proInclude`, a plain boolean). `proIncluded(it)` falls back to the original type-based rule (scripture/illustration only) whenever `proInclude` is unset, so every existing sermon's export is unchanged until a user explicitly touches an item's toggle.</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>Verified with Playwright: default on/off states match the old type-based rule exactly; manual overrides in either direction persist through save-and-reopen and are visible in the raw stored data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add tickets #67-68: print margin root-cause correction, Library rename
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J70" headerRowCount="1">
-  <autoFilter ref="A4:J70"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J72" headerRowCount="1">
+  <autoFilter ref="A4:J72"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3988,6 +3988,106 @@
       <c r="J70" s="5" t="inlineStr">
         <is>
           <t>Verified with Playwright: default on/off states match the old type-based rule exactly; manual overrides in either direction persist through save-and-reopen and are visible in the raw stored data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="100" customHeight="1">
+      <c r="A71" s="7" t="n">
+        <v>67</v>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>Prepare/Export</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Correct root cause of manuscript print margins; remove @page size:letter</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>User's screenshots proved #64's theory wrong: it's Chrome/Edge's own print preview the whole time (a "Print using system dialog" link is visible at the bottom of the same flyout), not a fallback to a bare OS dialog. The real issue is the dialog's "Margins" preset defaulting to "None" instead of "Default" -- manually switching it to Default produced exactly the intended layout. User asked directly whether this is something the app can influence.</t>
+        </is>
+      </c>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>Which Margins preset (Default vs None) the browser's print dialog opens on is a browser-remembered/sticky setting from past print jobs -- there is no CSS or JS mechanism to select it from web content. @page{margin:1in} only defines what "Default" means once chosen; it can't force that choice.</t>
+        </is>
+      </c>
+      <c r="G71" s="8" t="inlineStr">
+        <is>
+          <t>Removed the @page{size:letter} rule (kept only margin:1in), since forcing Letter against a destination printer/driver whose own configured page size differs is a plausible reason a browser falls back to "None" rather than computing "Default" against a mismatched page box. Not a guaranteed fix (unverifiable without the user's exact printer/driver) -- flagged honestly as removing one plausible contributing mismatch, not a certain resolution.</t>
+        </is>
+      </c>
+      <c r="H71" s="12" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
+        </is>
+      </c>
+      <c r="I71" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J71" s="8" t="inlineStr">
+        <is>
+          <t>User's own manual fix (switching Margins to Default) should persist going forward regardless, since Chrome remembers the last-used print setting across documents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="100" customHeight="1">
+      <c r="A72" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Add double-click-to-rename on Library sermon card titles</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>User: "let's also add the ability to edit a sermon name from the library screen. Make it so we arent accidentally doing this and try to accomplish it without adding a new button."</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>No way existed to rename a sermon without opening the full editor, and the user specifically wanted it discoverable from the Library card itself, without a new button and without risk of an accidental single-tap triggering it.</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>Double-click the title (the same convention as renaming a file in Finder/Explorer) swaps it for an inline, pre-filled, auto-selected input. Enter or blur commits (empty/unchanged values revert rather than save); Escape always reverts. A single click does nothing to it. Updates updatedAt and re-renders through the normal Library path, so a rename can reposition the sermon within its series group under Recent sort exactly like an editor-made edit would.</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>Verified with Playwright: single click never opens the input; double-click opens it pre-filled/focused; Enter commits and persists; Escape and empty-blur both revert without saving.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ticket #69: revert Library to flat by-sermon view
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -303,8 +303,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J72" headerRowCount="1">
-  <autoFilter ref="A4:J72"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J73" headerRowCount="1">
+  <autoFilter ref="A4:J73"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4088,6 +4088,56 @@
       <c r="J72" s="5" t="inlineStr">
         <is>
           <t>Verified with Playwright: single click never opens the input; double-click opens it pre-filled/focused; Enter commits and persists; Escape and empty-blur both revert without saving.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="90" customHeight="1">
+      <c r="A73" s="7" t="n">
+        <v>69</v>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>Library</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>Revert Library to flat by-sermon view (keep No-Series filter + rename)</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>User tried the series-grouped collapsible Library (#65) with real data and asked to revert it back to the by-sermon view.</t>
+        </is>
+      </c>
+      <c r="F73" s="8" t="inlineStr">
+        <is>
+          <t>Not a defect -- a UX preference reversal after hands-on evaluation. The grouped view was tried and judged not an improvement over the flat list.</t>
+        </is>
+      </c>
+      <c r="G73" s="8" t="inlineStr">
+        <is>
+          <t>Reverted the view only: renderLibrary() is back to the flat Recent / By-Date (Upcoming + Past-Undated) list; removed the collapsible group CSS, expand-state, and grouping helpers. Deliberately kept two things #65 introduced that don't depend on grouping: the "No Series" filter option in both Library and Plan slicers, and the double-click-to-rename on cards (#68).</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I73" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J73" s="8" t="inlineStr">
+        <is>
+          <t>The No-Series filter capability and inline rename were flagged to the user as kept-on-purpose rather than silently dropped with the view.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Triage backlog: file 5 user items to tracker (#70-73) + roadmap risks
- #70 ProPresenter on-site export test (Open)
- #71 import testing + example-sermon fixture (Open)
- #72 preferred Bible version setting (Parked; flagged as net-new feature)
- #73 dogfood real sermons on all devices (Open)
- Roadmap: add small-screen worth-$20 risk + parked feature to parking lot

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -91,8 +91,14 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="005B2A86"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -134,6 +140,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAD7F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -161,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -225,6 +236,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -303,8 +317,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J73" headerRowCount="1">
-  <autoFilter ref="A4:J73"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J77" headerRowCount="1">
+  <autoFilter ref="A4:J77"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -610,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4138,6 +4152,206 @@
       <c r="J73" s="8" t="inlineStr">
         <is>
           <t>The No-Series filter capability and inline rename were flagged to the user as kept-on-purpose rather than silently dropped with the view.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="100" customHeight="1">
+      <c r="A74" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Prepare/Export</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Field-test ProPresenter exports on-site at the church</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>User: "Test ProPresenter Exports (need to be at the church building for this). Allow ample time so I don't need to make multiple trips." The exported file needs to be opened in the actual ProPresenter install on the booth machine and driven through a real service flow, not just validated structurally on a dev box.</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>Plan: before the trip, lock down the export format and the per-item proInclude tagging so the file is known-good on paper; take a checklist to the building (import the file, confirm slide order/section breaks, confirm only pro-tagged items came through, project one live). Investigate whether a free ProPresenter trial or a second/duplicate license can be installed off-site so future export validation doesn't require a physical trip to the booth.</t>
+        </is>
+      </c>
+      <c r="H74" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>Batch every export question into one trip. Real-device / on-site, so it can only close after the church visit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="100" customHeight="1">
+      <c r="A75" s="7" t="n">
+        <v>71</v>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>Library/Import</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>Thoroughly test import on each device; author richer example sermons</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>User: "Thoroughly test import function, have claude write more fleshed-out example sermons to test well on each device." Current test data is thin; import needs to be exercised with realistic, full-length sermons (multiple sections, scripture, illustrations, formatting) on every target device.</t>
+        </is>
+      </c>
+      <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G75" s="8" t="inlineStr">
+        <is>
+          <t>Plan: I write a set of full, realistic sermons in the app's import/backup JSON format (varied series, section types, long manuscript bodies, pro-tagged and untagged items) as a reusable test fixture; user imports that fixture on each device and confirms round-trip fidelity (formatting, series, sections, pro tags, dates). I can produce the fixture on request.</t>
+        </is>
+      </c>
+      <c r="H75" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I75" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J75" s="8" t="inlineStr">
+        <is>
+          <t>Depends on me for the fixture, then user for the per-device import runs. Serves M1 / polish gate. No blasphemous or offensive content in the sample sermons.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="100" customHeight="1">
+      <c r="A76" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>Preferred Bible version setting that steers Blue Letter Bible lookups</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>User: "Add preferred bible version in settings page that determines where lookup sends to BLB search." A translation preference stored in settings would append the chosen version to the Blue Letter Bible search URL so lookups open in the pastor's preferred translation.</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>PARKED, not built. Flagged under the accountability deal: this is net-new feature scope, not on M1, M2, the polish gate, or M3. It is a small, genuinely reasonable papercut fix (many pastors have a fixed translation) and a fair candidate for the one-sitting wince-list once the polish gate opens -- but it should not be built ahead of the Mac build and the store signups. Revisit during the polish gate or post-M3.</t>
+        </is>
+      </c>
+      <c r="H76" s="24" t="inlineStr">
+        <is>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>Low effort when the time comes: settings-stored version code + query param on the existing BLB lookup URL. Confirm before building.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="100" customHeight="1">
+      <c r="A77" s="7" t="n">
+        <v>73</v>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>Dogfooding</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>Write real sermons in Shema on all devices</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>User: "Write a bunch of sermons in this thing on all devices." First-party real usage across phone/tablet/desktop, not synthetic test data.</t>
+        </is>
+      </c>
+      <c r="F77" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G77" s="8" t="inlineStr">
+        <is>
+          <t>This IS the polish-gate validation, not a side task: sustained real use is what surfaces the wince-items (and answers the small-screen value question, ticket-linked below). Plan: user drafts genuine sermons across every device during the polish window (Jul 23 - ~31); friction, layout problems, and any 'a pastor would notice this' issues get captured onto the single wince-list.</t>
+        </is>
+      </c>
+      <c r="H77" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I77" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J77" s="8" t="inlineStr">
+        <is>
+          <t>Directly feeds the polish gate and the small-screen worth-$20 risk on the roadmap. User-run.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add preferred Bible version setting (#72) + sample-sermon import fixture (#71)
- Settings > Bible Version select (15 BLB translations); lookup appends &t=<code>
- getBibleVersion() helper, localStorage-backed, defaults to KJV (BLB default = no-op)
- test-fixtures/shema-sample-sermons.json: 5 sermons/3 illustrations/39 items for
  import + dogfood testing across devices
- Verified via Playwright: default/persist/reload, full import, lookup URL threading
- Bump sw.js cache v92 -> v93

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -4186,7 +4186,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>Plan: before the trip, lock down the export format and the per-item proInclude tagging so the file is known-good on paper; take a checklist to the building (import the file, confirm slide order/section breaks, confirm only pro-tagged items came through, project one live). Investigate whether a free ProPresenter trial or a second/duplicate license can be installed off-site so future export validation doesn't require a physical trip to the booth.</t>
+          <t>Workaround researched. There is NO separate 'watermarked version' to find: ProPresenter 7 is a single free download that runs fully-featured in the EDITOR while unregistered; the watermark appears only on AUDIENCE/PROJECTION output, and only until licensed. The 2-week trial is a separate in-app request whose only purpose is removing that output watermark -- exactly what the user wants to reserve for live-projection marketing screenshots. Import validation never touches audience output, so it never triggers the watermark and never needs the trial: install the free version now, validate in the editor, keep the trial untouched. Also: the RTF export opens in Word/TextEdit/LibreOffice/Google Docs, so content, section breaks, scripture highlighting, and proInclude filtering can all be pre-validated at a desk -- reserving the church trip only for confirming ProPresenter's own slide segmentation on import.</t>
         </is>
       </c>
       <c r="H74" s="11" t="inlineStr">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="J74" s="5" t="inlineStr">
         <is>
-          <t>Batch every export question into one trip. Real-device / on-site, so it can only close after the church visit.</t>
+          <t>Still Open: the on-site slide-segmentation check requires the booth machine. Everything else is now doable off-site. Batch remaining export questions into the one trip.</t>
         </is>
       </c>
     </row>
@@ -4236,12 +4236,12 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>Plan: I write a set of full, realistic sermons in the app's import/backup JSON format (varied series, section types, long manuscript bodies, pro-tagged and untagged items) as a reusable test fixture; user imports that fixture on each device and confirms round-trip fidelity (formatting, series, sections, pro tags, dates). I can produce the fixture on request.</t>
-        </is>
-      </c>
-      <c r="H75" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Built the fixture: test-fixtures/shema-sample-sermons.json, a real Shema backup with 5 full sermons (2 named series + 1 No-Series), 3 illustrations, 39 items covering all four item types, rich text, 8 scripture refs, an explicit mix of proInclude true/false (12/3), and past+upcoming dates. Warm, orthodox, non-offensive content. Authored at current schemaVersion (sermon v2 / illustration v1) so import runs the identity path. User takes this to each device to test import.</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I75" s="8" t="inlineStr">
@@ -4251,7 +4251,7 @@
       </c>
       <c r="J75" s="8" t="inlineStr">
         <is>
-          <t>Depends on me for the fixture, then user for the per-device import runs. Serves M1 / polish gate. No blasphemous or offensive content in the sample sermons.</t>
+          <t>Import verified with Playwright (5 sermons/3 illustrations/39 items, all types, both proInclude states, all series incl. No-Series, all titles rendered). Per-device human import runs on real hardware still pending -- that half stays with the user.</t>
         </is>
       </c>
     </row>
@@ -4286,12 +4286,12 @@
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>PARKED, not built. Flagged under the accountability deal: this is net-new feature scope, not on M1, M2, the polish gate, or M3. It is a small, genuinely reasonable papercut fix (many pastors have a fixed translation) and a fair candidate for the one-sitting wince-list once the polish gate opens -- but it should not be built ahead of the Mac build and the store signups. Revisit during the polish gate or post-M3.</t>
-        </is>
-      </c>
-      <c r="H76" s="24" t="inlineStr">
-        <is>
-          <t>Parked</t>
+          <t>Built. Added a Bible Version &lt;select&gt; to Settings (between Restore and Dark Mode) with the 15 common English translations BLB serves via its t= search parameter (KJV, NKJV, ESV, NIV, NLT, CSB, NASB20, NASB95, LSB, AMP, NET, RSV, ASV, YLT, WEB). Stored in localStorage via a hoisted getBibleVersion() helper (default KJV = BLB's own default, so untouched = no change); the scripture-lookup handler appends &amp;t=&lt;code&gt; to the BLB URL when set. User acknowledged the net-new-feature flag and green-lit it as off-critical-path and low-cost.</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I76" s="5" t="inlineStr">
@@ -4301,7 +4301,7 @@
       </c>
       <c r="J76" s="5" t="inlineStr">
         <is>
-          <t>Low effort when the time comes: settings-stored version code + query param on the existing BLB lookup URL. Confirm before building.</t>
+          <t>Verified with Playwright: defaults to KJV, ESV selection persists across reload, and a real lookup click opened ...&amp;t=ESV. Off the M2 critical path, so building it now cost no schedule.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Native .docx import + per-paragraph block splitting (#74)
- Upload File now accepts .docx: hand-parse the ZIP + inflate via native
  DecompressionStream (no libraries, CSP-safe), then map document.xml to
  import HTML (headings->section breaks, paragraphs->blocks, b/i/u, lists
  from numbering.xml, tables->row-joined lines)
- Fix monolith-block bug for all imports: importStagingToSections splits into
  one block per paragraph at top-level <br> boundaries
- Feature-detect DecompressionStream with graceful fallback; update accept +
  modal help text
- Verified all five Word sample docs via Playwright; bump sw.js v93 -> v94

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -317,8 +317,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J77" headerRowCount="1">
-  <autoFilter ref="A4:J77"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J78" headerRowCount="1">
+  <autoFilter ref="A4:J78"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4352,6 +4352,56 @@
       <c r="J77" s="8" t="inlineStr">
         <is>
           <t>Directly feeds the polish gate and the small-screen worth-$20 risk on the roadmap. User-run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="120" customHeight="1">
+      <c r="A78" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Library/Import</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Native .docx upload + per-paragraph block splitting on import</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>User tested the Word paste-samples and found (a) uploading a .docx via 'Upload File' dumped raw ZIP bytes ('PK...') because the handler only readAsText'd it, and (b) pasting a manuscript produced one giant undifferentiated block. The iPad/write-in-Word-then-paste pastor is the core reason this path exists, so the user chose the full fix over graceful-degradation-only.</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>Upload handler only ever read files as text, so a .docx (a ZIP) came through as binary. Separately, importStagingToSections collapsed everything between section-break markers into a single 'block' item, so prose with no Word headings became one monolith.</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>Built native in-app .docx parsing with NO libraries: hand-parse the ZIP central directory and inflate DEFLATE entries with the platform's own DecompressionStream('deflate-raw') (CSP-safe, no external host/eval); parse word/document.xml + numbering.xml with DOMParser. Word Heading/Title paragraphs -&gt; section-break markers; every other paragraph -&gt; its own block; w:b/w:i/w:u -&gt; strong/em/u (off values respected); numbered vs bulleted lists read from numbering.xml; tables degrade to one row-joined line each. Upload handler branches on .docx, feature-detects DecompressionStream (friendly fallback toast if absent), and shows clear errors. ALSO fixed the monolith bug for all imports (paste included): importStagingToSections now splits into one block per paragraph at top-level &lt;br&gt; boundaries (blank lines collapse; a whole list stays one block). Updated file-input accept + modal help text.</t>
+        </is>
+      </c>
+      <c r="H78" s="12" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>Verified with Playwright on all five sample docs (DecompressionStream present in-engine, no page errors, correct sections/blocks/lists, table degraded to readable row-joined blocks, no empty blocks, no lost words). Needs on-device confirmation: (1) DecompressionStream('deflate-raw') needs a modern WebView (Chromium 80+/iOS 16.4+) -- feature-detected but confirm on target; (2) heading detection keys off the style id (Heading1..9/Title/Subtitle), may miss localized/oddly-named custom styles.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log #75: native Google/email-link sign-in strands session in Safari
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -317,8 +317,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J78" headerRowCount="1">
-  <autoFilter ref="A4:J78"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J79" headerRowCount="1">
+  <autoFilter ref="A4:J79"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J78"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4402,6 +4402,56 @@
       <c r="J78" s="5" t="inlineStr">
         <is>
           <t>Verified with Playwright on all five sample docs (DecompressionStream present in-engine, no page errors, correct sections/blocks/lists, table degraded to readable row-joined blocks, no empty blocks, no lost words). Needs on-device confirmation: (1) DecompressionStream('deflate-raw') needs a modern WebView (Chromium 80+/iOS 16.4+) -- feature-detected but confirm on target; (2) heading detection keys off the style id (Heading1..9/Title/Subtitle), may miss localized/oddly-named custom styles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="130" customHeight="1">
+      <c r="A79" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>Account/Auth</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>Native app: Google + email-link sign-in completes in Safari, not in the app</t>
+        </is>
+      </c>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>Found during M1 on-device testing: tapping Continue with Google opens Safari, sign-in succeeds there, but the session never returns to the app. Same latent flaw affects the email magic-link button.</t>
+        </is>
+      </c>
+      <c r="F79" s="8" t="inlineStr">
+        <is>
+          <t>signInWithOAuth/signInWithOtp use redirectTo = window.location.origin+pathname. In the native WebView that resolves to the app's internal localhost, which the external browser can't hand control back to -- so Supabase's post-auth redirect lands in Safari, stranding the session outside the app. No deep-link scheme, no appUrlOpen listener, no PKCE code exchange exist yet.</t>
+        </is>
+      </c>
+      <c r="G79" s="8" t="inlineStr">
+        <is>
+          <t>PLAN (not built): native branch using a custom-scheme deep link. (1) app code: on native set redirectTo=com.shema.app://auth-callback, skipBrowserRedirect:true, open the URL via @capacitor/browser, add @capacitor/app appUrlOpen listener -&gt; exchangeCodeForSession -&gt; refresh UI; set flowType:'pkce'. (2) native config: CFBundleURLTypes in iOS Info.plist + Android intent filter for the scheme. (3) add @capacitor/app + @capacitor/browser plugins. (4) USER: add the deep-link URL to Supabase Auth &gt; URL Configuration &gt; Redirect URLs. (5) rebuild + device retest. Fixes Google AND email-link. Can't be fully verified off-device (needs live Supabase + real device).</t>
+        </is>
+      </c>
+      <c r="H79" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I79" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J79" s="8" t="inlineStr">
+        <is>
+          <t>NOT blocking the pastor beta: sign-in is only for cross-device sync (paid feature); the whole app works offline with no account. Must fix before selling sync. Native Google Sign-In SDK (signInWithIdToken) is a possible later UX upgrade but email-link still needs the deep-link path, so deep-link is the right foundation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log device bugs #76-78 + parked scripture-tool #79; note Apple enrollment done
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -317,8 +317,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J79" headerRowCount="1">
-  <autoFilter ref="A4:J79"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J83" headerRowCount="1">
+  <autoFilter ref="A4:J83"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4452,6 +4452,206 @@
       <c r="J79" s="8" t="inlineStr">
         <is>
           <t>NOT blocking the pastor beta: sign-in is only for cross-device sync (paid feature); the whole app works offline with no account. Must fix before selling sync. Native Google Sign-In SDK (signInWithIdToken) is a possible later UX upgrade but email-link still needs the deep-link path, so deep-link is the right foundation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="115" customHeight="1">
+      <c r="A80" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Library/UI</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Sermon title clipped on the sermon-details screen</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>Device report (M1 testing): the sermon title is cut off / clipped on the sermon details (info) screen.</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>Likely a fixed-height or non-wrapping title element (overflow hidden / no line-height room) in the sermon info modal or the editor title display -- to confirm in code.</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>PLAN (not built): let the title wrap or ellipsize with room -- adjust the title element's overflow/white-space/line-height/height so the full title shows. Quick CSS fix.</t>
+        </is>
+      </c>
+      <c r="H80" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>Quick polish fix; batch with the other device bugs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="115" customHeight="1">
+      <c r="A81" s="7" t="n">
+        <v>77</v>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>Editor/Native</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>Rotating the device while typing leaves the text box hidden behind the keyboard</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>Device report (M1 testing): if screen orientation changes while entering text, the focused text box gets stuck behind the on-screen keyboard.</t>
+        </is>
+      </c>
+      <c r="F81" s="8" t="inlineStr">
+        <is>
+          <t>Native WebView doesn't re-scroll the focused field into view when the viewport reflows on orientation change; the keyboard then covers it.</t>
+        </is>
+      </c>
+      <c r="G81" s="8" t="inlineStr">
+        <is>
+          <t>PLAN (not built): on resize/orientationchange, scroll the focused input/contenteditable back into view (scrollIntoView); consider the Capacitor Keyboard plugin resize mode, and/or evaluate locking the phone UI to portrait (Present already benefits from a fixed orientation). More involved than a CSS tweak; verify on device.</t>
+        </is>
+      </c>
+      <c r="H81" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I81" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J81" s="8" t="inlineStr">
+        <is>
+          <t>Native-specific; needs on-device retest after fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="115" customHeight="1">
+      <c r="A82" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Chore</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Editor/Settings</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Remove text-based scripture lookup until a proper dedicated tool is built</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>User decision (M1 testing): scripture lookup shouldn't be driven by scraping whatever text is in the scripture item -- it should be a dedicated tool. Remove the current lookup for now so a half-formed feature isn't in front of pastors.</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>Current lookup (data-act=lookup) builds a Blue Letter Bible search URL from the scripture item's text -- not the intended model.</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>PLAN (not built): remove/hide the lookup button + its handler. DEPENDENCY: this orphans the Bible Version setting (#72), whose only job is steering this lookup -- so also hide that Settings row (keep the stored pref + getBibleVersion code dormant) and re-enable it when the proper tool (#79) ships. Flagged to user.</t>
+        </is>
+      </c>
+      <c r="H82" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>Quick removal; entangled with #72 -- confirm hiding the Bible Version setting too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="115" customHeight="1">
+      <c r="A83" s="7" t="n">
+        <v>79</v>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>Editor</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>Build a proper dedicated scripture lookup tool</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>Replacement for the removed text-based lookup (#78): a first-class tool where the user explicitly enters/《picks》a reference and translation and previews/inserts it, rather than scraping the scripture box text.</t>
+        </is>
+      </c>
+      <c r="F83" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G83" s="8" t="inlineStr">
+        <is>
+          <t>PARKED (future): design a dedicated lookup UI. When built, re-enable the Bible Version setting (#72), which was hidden in #78. Scope TBD -- online BLB deep-link vs. a bundled offline text (note: an offline KJV lookup was previously removed, #46, so revisit that decision deliberately).</t>
+        </is>
+      </c>
+      <c r="H83" s="24" t="inlineStr">
+        <is>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="I83" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J83" s="8" t="inlineStr">
+        <is>
+          <t>Re-enables #72 when done. Confirm scope before building.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 1 device fixes: title clip (#76), keyboard-on-rotation (#77), remove scripture lookup (#78)
- #78 (Done): remove text-based scripture Look up button + handler; hide the
  Bible Version settings row (keep getBibleVersion/select dormant for #79)
- #76 (Needs Testing): line-height on #titleInput so Playfair descenders don't
  clip in Sermon Details; noted the 15px-vs-19px specificity quirk, left size as-is
- #77 (Needs Testing): scroll focused field into view on visualViewport resize /
  orientationchange
- Bump sw.js v94 -> v95; verified in-browser, no page errors

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -4489,9 +4489,9 @@
           <t>PLAN (not built): let the title wrap or ellipsize with room -- adjust the title element's overflow/white-space/line-height/height so the full title shows. Quick CSS fix.</t>
         </is>
       </c>
-      <c r="H80" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="H80" s="12" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
         </is>
       </c>
       <c r="I80" s="5" t="inlineStr">
@@ -4501,7 +4501,7 @@
       </c>
       <c r="J80" s="5" t="inlineStr">
         <is>
-          <t>Quick polish fix; batch with the other device bugs.</t>
+          <t>Fix: added line-height:1.5 to #titleInput so Playfair's descenders aren't clipped in the Sermon Details modal. Verified in-browser (no clip room issue). NOTE: the title font resolves to 15px, not the intended 19px -- a higher-specificity #editorMeta input rule overrides #titleInput; left the size as-is (out of scope) and only fixed the clip. Confirm on device which title clipped (modal input vs the brandbar title button); redirect the fix if it was the top bar.</t>
         </is>
       </c>
     </row>
@@ -4539,9 +4539,9 @@
           <t>PLAN (not built): on resize/orientationchange, scroll the focused input/contenteditable back into view (scrollIntoView); consider the Capacitor Keyboard plugin resize mode, and/or evaluate locking the phone UI to portrait (Present already benefits from a fixed orientation). More involved than a CSS tweak; verify on device.</t>
         </is>
       </c>
-      <c r="H81" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="H81" s="12" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
         </is>
       </c>
       <c r="I81" s="8" t="inlineStr">
@@ -4551,7 +4551,7 @@
       </c>
       <c r="J81" s="8" t="inlineStr">
         <is>
-          <t>Native-specific; needs on-device retest after fix.</t>
+          <t>Fix: on visualViewport 'resize' and window 'orientationchange', scroll the focused input/textarea/contenteditable back into view (250ms settle, block:center). Harmless on web. Verified it parses with no errors; the behind-keyboard behavior itself is device-only -- confirm on the phone by rotating mid-typing.</t>
         </is>
       </c>
     </row>
@@ -4589,9 +4589,9 @@
           <t>PLAN (not built): remove/hide the lookup button + its handler. DEPENDENCY: this orphans the Bible Version setting (#72), whose only job is steering this lookup -- so also hide that Settings row (keep the stored pref + getBibleVersion code dormant) and re-enable it when the proper tool (#79) ships. Flagged to user.</t>
         </is>
       </c>
-      <c r="H82" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
@@ -4601,7 +4601,7 @@
       </c>
       <c r="J82" s="5" t="inlineStr">
         <is>
-          <t>Quick removal; entangled with #72 -- confirm hiding the Bible Version setting too.</t>
+          <t>Removed the scripture 'Look up' button + its handler; hid the Settings &gt; Bible Version row (display:none) and left getBibleVersion + the select dormant for #79. Verified: 0 lookup buttons render on a scripture item, the item still edits normally, and the settings row computes display:none.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Native deep-link auth for Google + email sign-in (#75)
Fixes sign-in stranding the session in Safari on the native app.
- index.html: native branch uses redirectTo=com.shema.app://auth-callback +
  skipBrowserRedirect, opens auth URL via @capacitor/browser, and an
  @capacitor/app appUrlOpen listener does exchangeCodeForSession to finish in
  the app; email magic-link uses the same deep link on native; client set to
  flowType:pkce + detectSessionInUrl:false on native only (web untouched)
- iOS Info.plist CFBundleURLTypes + Android intent-filter for com.shema.app
- package.json: add @capacitor/app + @capacitor/browser
- Bump sw.js v95 -> v96

Verified structurally in-browser (web unchanged, parses clean); native round-trip
needs on-device test + a Supabase redirect-URL setting.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -4405,7 +4405,7 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="130" customHeight="1">
+    <row r="79" ht="175" customHeight="1">
       <c r="A79" s="7" t="n">
         <v>75</v>
       </c>
@@ -4436,12 +4436,12 @@
       </c>
       <c r="G79" s="8" t="inlineStr">
         <is>
-          <t>PLAN (not built): native branch using a custom-scheme deep link. (1) app code: on native set redirectTo=com.shema.app://auth-callback, skipBrowserRedirect:true, open the URL via @capacitor/browser, add @capacitor/app appUrlOpen listener -&gt; exchangeCodeForSession -&gt; refresh UI; set flowType:'pkce'. (2) native config: CFBundleURLTypes in iOS Info.plist + Android intent filter for the scheme. (3) add @capacitor/app + @capacitor/browser plugins. (4) USER: add the deep-link URL to Supabase Auth &gt; URL Configuration &gt; Redirect URLs. (5) rebuild + device retest. Fixes Google AND email-link. Can't be fully verified off-device (needs live Supabase + real device).</t>
-        </is>
-      </c>
-      <c r="H79" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>BUILT (native deep-link flow). JS: native branch on Google sign-in uses redirectTo=com.shema.app://auth-callback + skipBrowserRedirect, opens the auth URL via @capacitor/browser (fallback window.open _system), and an @capacitor/app appUrlOpen listener exchanges the PKCE code (exchangeCodeForSession) to finish the session in-app; email magic-link uses the same deep-link emailRedirectTo on native; the Supabase client is created with flowType:pkce + detectSessionInUrl:false ONLY on native (web keeps defaults untouched). Native config: iOS Info.plist CFBundleURLTypes + Android intent-filter for the com.shema.app scheme. Deps: added @capacitor/app + @capacitor/browser to package.json.</t>
+        </is>
+      </c>
+      <c r="H79" s="12" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
         </is>
       </c>
       <c r="I79" s="8" t="inlineStr">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="J79" s="8" t="inlineStr">
         <is>
-          <t>NOT blocking the pastor beta: sign-in is only for cross-device sync (paid feature); the whole app works offline with no account. Must fix before selling sync. Native Google Sign-In SDK (signInWithIdToken) is a possible later UX upgrade but email-link still needs the deep-link path, so deep-link is the right foundation.</t>
+          <t>Verified structurally in-browser (parses clean on web+native mock, no page errors; web path unchanged; callback-URL parsing sound). The native round-trip CANNOT be verified off-device -- headless @capacitor/core reports platform 'web' so isNativePlatform() is false there. USER STEPS to finish: (1) npm install &amp;&amp; npm run sync (pulls the two new Capacitor plugins into the native project); (2) in Supabase Auth &gt; URL Configuration add redirect URL com.shema.app://auth-callback; (3) rebuild in Xcode and test Continue with Google + the email link on the phone -- both should now return into the app.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reframe #70 (time not hard-stop); research free-API scripture tool for #79
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -4186,7 +4186,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>Workaround researched. There is NO separate 'watermarked version' to find: ProPresenter 7 is a single free download that runs fully-featured in the EDITOR while unregistered; the watermark appears only on AUDIENCE/PROJECTION output, and only until licensed. The 2-week trial is a separate in-app request whose only purpose is removing that output watermark -- exactly what the user wants to reserve for live-projection marketing screenshots. Import validation never touches audience output, so it never triggers the watermark and never needs the trial: install the free version now, validate in the editor, keep the trial untouched. Also: the RTF export opens in Word/TextEdit/LibreOffice/Google Docs, so content, section breaks, scripture highlighting, and proInclude filtering can all be pre-validated at a desk -- reserving the church trip only for confirming ProPresenter's own slide segmentation on import.</t>
+          <t>Not a hard blocker -- just needs time. ProPresenter 7 is a single free download that runs fully featured in the EDITOR while unregistered (the watermark only touches live audience output, and only until licensed). So install the free version on the LAPTOP and validate Shema's RTF import there -- import the file, check slide order / section breaks / that only the pro-tagged items came through -- with no watermark and no church trip, keeping the 2-week trial untouched for marketing screenshots later. The RTF also opens in Word/TextEdit/LibreOffice/Google Docs for a quick content check. The physical booth visit is now OPTIONAL -- only for final confidence that PP on the actual service machine segments slides as expected; batch it into a normal trip, no special errand needed.</t>
         </is>
       </c>
       <c r="H74" s="11" t="inlineStr">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="J74" s="5" t="inlineStr">
         <is>
-          <t>Still Open: the on-site slide-segmentation check requires the booth machine. Everything else is now doable off-site. Batch remaining export questions into the one trip.</t>
+          <t>Downgraded from 'requires a church trip' to 'needs an unhurried hour on the laptop.' On-site check is a nice-to-have, not a gate.</t>
         </is>
       </c>
     </row>
@@ -4636,7 +4636,7 @@
       </c>
       <c r="G83" s="8" t="inlineStr">
         <is>
-          <t>PARKED (future): design a dedicated lookup UI. When built, re-enable the Bible Version setting (#72), which was hidden in #78. Scope TBD -- online BLB deep-link vs. a bundled offline text (note: an offline KJV lookup was previously removed, #46, so revisit that decision deliberately).</t>
+          <t>FEASIBLE with free, keyless APIs -- and it can be genuinely more functional than the old link-out. Design (not built): a dedicated lookup tool where the user types/confirms a reference (e.g. 'John 3:16', 'Rom 8:28-30'), the app fetches the passage from a free no-key public-domain API (bible-api.com or the AO Lab 'Free Use Bible API' at bible.helloao.org -- both keyless, CORS, no usage limits), shows the text in a panel, and offers Insert-as-scripture-item / Copy. Re-enables the Bible Version setting (#72) for the translation picker. LICENSING CAVEAT (the catch): only PUBLIC-DOMAIN translations (KJV, ASV, WEB, YLT, Darby, BBE) can be displayed in-app for free -- those are unrestricted even commercially. Modern copyrighted translations (ESV, NIV, NASB, CSB) CANNOT be shown as full text in a PAID app for free: API.Bible's free tier is non-commercial only, and ESV/Crossway licenses to organizations, not solo devs. So for copyrighted versions, fall back to a labeled 'open in Blue Letter Bible' link-out (the old behavior, but now a deliberate secondary path). TECH: needs the API host added to the CSP connect-src (ties into #29); lookup needs network so degrade gracefully offline (or optionally bundle a PD KJV for offline -- note #46 removed an offline KJV before, so revisit that deliberately).</t>
         </is>
       </c>
       <c r="H83" s="24" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="J83" s="8" t="inlineStr">
         <is>
-          <t>Re-enables #72 when done. Confirm scope before building.</t>
+          <t>PARKED / off the beta critical path (net-new feature, not M1/M2/polish/M3). Strictly better than the old search-link for PD translations. Confirm scope before building; realistic slot is during polish or post-beta. Sources: bible-api.com, bible.helloao.org (Free Use Bible API), scripture.api.bible (non-commercial only), api.esv.org (org license only).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Responsiveness audit (#42): clean; fix illustration tags-not-array crash (#80)
- Audited 5 viewports x 8 views/modals via Playwright: zero horizontal overflow,
  all tap targets >=40px. No layout fixes needed.
- #80: coerce illustration tags to an array in normalizeIllustration (string ->
  comma-split like the editor; non-array -> []) so a comma-string from an old
  backup or imported JSON no longer crashes the Illustrations view (.map/.some/.join)
- Correct the sample-sermons.json fixture (illustration tags were strings)
- Bump sw.js v96 -> v97

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -317,8 +317,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J83" headerRowCount="1">
-  <autoFilter ref="A4:J83"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J84" headerRowCount="1">
+  <autoFilter ref="A4:J84"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2786,12 +2786,12 @@
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>Fixed .line missing overflow-wrap (long words clipping on Present/Practice stage text).</t>
-        </is>
-      </c>
-      <c r="H46" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Ran an automated cross-viewport audit (Playwright): 5 viewports -- 320px phone, 393px phone, phone landscape (852x393), iPad portrait 768, iPad landscape 1024 -- across Library, Plan, Illustrations, Prepare/editor, Present, and the Settings/Import/Sermon-Details modals. Measured page-level horizontal overflow + any element crossing the viewport edge, and interactive-target sizes on phones. RESULT: zero horizontal overflow anywhere; all tap targets &gt;= 40px on both phone sizes. Responsiveness is clean -- the earlier mobile passes (#41, #56-58) hold up. The audit ALSO surfaced a real crash (illustration string-tags) -&gt; fixed as #80.</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I46" s="8" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="J46" s="8" t="inlineStr">
         <is>
-          <t>~50 flagged items from the corrected re-run were never fully triaged -- deprioritized in favor of the user's punch list.</t>
+          <t>Done via automated harness. Caveat: this covers layout/overflow + tap sizes objectively, not pixel-level visual polish or real-device rendering quirks -- those stay with your on-device beta pass (the title-clip #76 and keyboard #77 are already tracked separately). No overflow fixes were needed.</t>
         </is>
       </c>
     </row>
@@ -4652,6 +4652,56 @@
       <c r="J83" s="8" t="inlineStr">
         <is>
           <t>PARKED / FLAGGED -- no solid fix. Decision (2026-07-23): the old lookup's genuine value was BLB KEYWORD/WORD searches (finding everywhere a word or phrase appears), not reference lookups -- and that word-search use case has no clean fix under the only licensing-safe model we have (link out -&gt; user copies text back), since in-app text display is ruled out by cost/licensing. A reference-aware link-out (Bible Gateway passage URL + book/chapter/verse picker + plain-text paste) was designed (see Fix/Resolution) and would handle passage lookups well, but it doesn't recreate the word-search strength that made the old tool nice. Net: not worth building now; net-new feature, off the beta critical path. Leaving removed (#78 stands) and parked until it clearly earns its place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="115" customHeight="1">
+      <c r="A84" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Illustrations</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Illustrations view crashes when an illustration's tags aren't an array</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>Surfaced by the #42 responsiveness audit: loading/importing an illustration whose tags is a comma-string (not an array) throws '(ill.tags||[]).map is not a function' and breaks the Illustrations view + search.</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>Render (itags .map), search (.some), and the edit form (.join) all treat ill.tags as an array, and the ||[] guard only catches null/undefined -- a truthy string slips through and .map/.some/.join throw. normalizeIllustration did no shape coercion (unlike normalizeSermon).</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>Coerce tags to an array in normalizeIllustration (runs on both load and import): a string is comma-split/trimmed/filtered exactly like the editor does on save; any other non-array becomes []. Also corrected the sample-sermons.json import fixture, whose illustrations had string tags and would have crashed Illustrations on import.</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>Verified with the audit harness: after the fix, no page errors on the Illustrations view at any viewport, and tags render as chips. Bumped sw.js v96 -&gt; v97.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log #81: post-launch smart-watch Present-timer companion (parked)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -317,8 +317,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J84" headerRowCount="1">
-  <autoFilter ref="A4:J84"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J85" headerRowCount="1">
+  <autoFilter ref="A4:J85"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4702,6 +4702,56 @@
       <c r="J84" s="5" t="inlineStr">
         <is>
           <t>Verified with the audit harness: after the fix, no page errors on the Illustrations view at any viewport, and tags render as chips. Bumped sw.js v96 -&gt; v97.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="105" customHeight="1">
+      <c r="A85" s="7" t="n">
+        <v>81</v>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>Smart-watch companion: show the Present countdown timer on the wrist</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>POST-LAUNCH idea (user): during Present, mirror the sermon countdown timer to the pastor's Apple Watch / Wear OS watch, so they can glance at remaining time on their wrist instead of looking down at the phone/podium.</t>
+        </is>
+      </c>
+      <c r="F85" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G85" s="8" t="inlineStr">
+        <is>
+          <t>PARKED / post-launch. Note: this is real native work beyond the Capacitor WebView -- watchOS and Wear OS companions are separate native targets (SwiftUI / Kotlin) with their own build + store steps, not something the shared HTML app can do on its own. Scope carefully; likely a v2 / premium-tier feature. Pairs with the distraction-free-presenting theme (we already keep the screen awake during Present via navigator.wakeLock).</t>
+        </is>
+      </c>
+      <c r="H85" s="24" t="inlineStr">
+        <is>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="I85" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J85" s="8" t="inlineStr">
+        <is>
+          <t>Explicitly post-launch, off the beta critical path. Logged per user request; revisit after M3/M4.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
#75 native sign-in confirmed on device -> Done (fix was the Supabase redirect URL)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -4439,9 +4439,9 @@
           <t>BUILT (native deep-link flow). JS: native branch on Google sign-in uses redirectTo=com.shema.app://auth-callback + skipBrowserRedirect, opens the auth URL via @capacitor/browser (fallback window.open _system), and an @capacitor/app appUrlOpen listener exchanges the PKCE code (exchangeCodeForSession) to finish the session in-app; email magic-link uses the same deep-link emailRedirectTo on native; the Supabase client is created with flowType:pkce + detectSessionInUrl:false ONLY on native (web keeps defaults untouched). Native config: iOS Info.plist CFBundleURLTypes + Android intent-filter for the com.shema.app scheme. Deps: added @capacitor/app + @capacitor/browser to package.json.</t>
         </is>
       </c>
-      <c r="H79" s="12" t="inlineStr">
-        <is>
-          <t>Needs Testing</t>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I79" s="8" t="inlineStr">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="J79" s="8" t="inlineStr">
         <is>
-          <t>Verified structurally in-browser (parses clean on web+native mock, no page errors; web path unchanged; callback-URL parsing sound). The native round-trip CANNOT be verified off-device -- headless @capacitor/core reports platform 'web' so isNativePlatform() is false there. USER STEPS to finish: (1) npm install &amp;&amp; npm run sync (pulls the two new Capacitor plugins into the native project); (2) in Supabase Auth &gt; URL Configuration add redirect URL com.shema.app://auth-callback; (3) rebuild in Xcode and test Continue with Google + the email link on the phone -- both should now return into the app.</t>
+          <t>CONFIRMED ON DEVICE (2026-07-23). Root of the last-mile issue: the com.shema.app://auth-callback redirect URL was not in Supabase Auth &gt; URL Configuration &gt; Redirect URLs, so Supabase fell back to the Site URL (logged in inside the in-app browser, never handed back to the app). After the user added that redirect URL, Google sign-in returns into the app logged in. Email magic-link uses the same redirect + handler.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Force Google account picker (#82); diagnose magic-link deep-link + branding (#83)
- #82: add queryParams:{prompt:'select_account'} to signInWithOAuth (native +
  web) so Google always shows the account chooser instead of silently reusing
  an existing session
- #83 (open, not code): diagnosed magic-link failing to return to the app as
  an in-app-browser custom-scheme limitation (mail apps commonly block the
  final redirect hop); workaround is opening the link in Safari. Robust fix
  needs Universal Links + a domain. Also: default Supabase email templates
  are unbranded -- fix is dashboard-side (Auth > Email Templates)
- Bump sw.js v97 -> v98

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -317,8 +317,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J85" headerRowCount="1">
-  <autoFilter ref="A4:J85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J87" headerRowCount="1">
+  <autoFilter ref="A4:J87"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4752,6 +4752,106 @@
       <c r="J85" s="8" t="inlineStr">
         <is>
           <t>Explicitly post-launch, off the beta critical path. Logged per user request; revisit after M3/M4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="190" customHeight="1">
+      <c r="A86" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Account/Auth</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>Native Google sign-in never showed the account picker</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>User (device testing): Continue with Google went straight to whichever Google account was already signed into the device, with no chance to pick a different one.</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>Google's OAuth endpoint silently reuses any existing session in the browser context (the in-app browser shares Safari's cookie store on iOS), and defaults to skipping the account chooser when exactly one session is present -- NOT an unavoidable platform limitation, just a missing OAuth parameter.</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>FIXED. Added queryParams:{prompt:'select_account'} to the signInWithOAuth call (both native and web branches) -- forwarded straight to Google's own authorize endpoint, forces the account picker on every sign-in regardless of an existing session.</t>
+        </is>
+      </c>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>Verified: parses clean, no page errors, correct object-spread syntax (options:{redirectTo, skipBrowserRedirect, ...queryParams}). The actual picker UI can only be confirmed on a real device against live Google OAuth -- same limitation as #75's native round-trip. Bumped sw.js v97 -&gt; v98.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="190" customHeight="1">
+      <c r="A87" s="7" t="n">
+        <v>83</v>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>Account/Auth</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>Email magic-link sign-in doesn't return to the native app; link is unbranded (raw Supabase URL)</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>User (device testing): sent a magic link to a Yahoo address, tapped it, and was not returned to / logged into the app. Separately, the email itself shows no Shema branding -- just a raw Supabase URL.</t>
+        </is>
+      </c>
+      <c r="F87" s="8" t="inlineStr">
+        <is>
+          <t>TWO separate root causes. (1) Return-to-app failure: the magic link is opened by an EXTERNAL, uncontrolled context (whatever browser the Yahoo/Mail app embeds), unlike Google sign-in which we open ourselves via @capacitor/browser. Many mail-app in-app browsers block/ignore the final redirect hop from Supabase's https://...supabase.co/auth/v1/verify link to our custom URL scheme (com.shema.app://auth-callback) as a phishing precaution -- custom schemes require the browser itself to hand off to the OS, and many mail-app browsers refuse to for exactly this class of link. (2) Branding: Supabase's built-in Auth email templates are unbranded by default -- the magic-link email shows the raw project verify URL as the link text, with no Shema name/styling.</t>
+        </is>
+      </c>
+      <c r="G87" s="8" t="inlineStr">
+        <is>
+          <t>NOT YET FIXED -- dashboard-side work, not app code. (1) Immediate workaround: open the emailed link via 'Open in Safari' / the system browser instead of the mail app's built-in one -- Safari respects the custom-scheme handoff (this is exactly how Google sign-in already works). ROBUST fix: switch native magic-link redirect from the com.shema.app:// custom scheme to a Universal Link (a real https:// URL on a domain we control, with an apple-app-site-association file + the Associated Domains capability in Xcode) -- iOS intercepts Universal Links at the OS level before any browser loads them, so restrictive mail-app browsers can't block the handoff. Needs a domain (none currently configured for this beyond the in-app marketing page) -- confirm with user whether one exists/should be acquired. (2) Edit Authentication &gt; Email Templates &gt; Magic Link in the Supabase dashboard: change subject + body copy to say 'Shema', give the link friendly anchor text ('Open in Shema') instead of a bare URL. Also flagged: Supabase's default built-in email sender has a low rate limit (dev/testing tier) -- worth Custom SMTP (Resend/Postmark/etc.) before many pastors test magic-link sign-in around the same time, which fixes branding AND the rate limit together.</t>
+        </is>
+      </c>
+      <c r="H87" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I87" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J87" s="8" t="inlineStr">
+        <is>
+          <t>Recommend for the beta: tell pastors to use Continue with Google if possible (fully working), or open magic-link emails via 'Open in Safari' if they hit this. Full Universal Links fix and/or Custom SMTP are real but non-trivial follow-ups -- scope with user before building.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Split #83 (parked, needs domain) from #84 (email branding, ready to paste)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -172,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -239,6 +239,9 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -317,8 +320,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J87" headerRowCount="1">
-  <autoFilter ref="A4:J87"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tickets" displayName="Tickets" ref="A4:J88" headerRowCount="1">
+  <autoFilter ref="A4:J88"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Type"/>
@@ -624,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4805,7 +4808,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="190" customHeight="1">
+    <row r="87" ht="145" customHeight="1">
       <c r="A87" s="7" t="n">
         <v>83</v>
       </c>
@@ -4819,9 +4822,9 @@
           <t>Account/Auth</t>
         </is>
       </c>
-      <c r="D87" s="8" t="inlineStr">
-        <is>
-          <t>Email magic-link sign-in doesn't return to the native app; link is unbranded (raw Supabase URL)</t>
+      <c r="D87" s="25" t="inlineStr">
+        <is>
+          <t>Magic-link sign-in doesn't return to the native app (custom-scheme limitation)</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
@@ -4836,12 +4839,12 @@
       </c>
       <c r="G87" s="8" t="inlineStr">
         <is>
-          <t>NOT YET FIXED -- dashboard-side work, not app code. (1) Immediate workaround: open the emailed link via 'Open in Safari' / the system browser instead of the mail app's built-in one -- Safari respects the custom-scheme handoff (this is exactly how Google sign-in already works). ROBUST fix: switch native magic-link redirect from the com.shema.app:// custom scheme to a Universal Link (a real https:// URL on a domain we control, with an apple-app-site-association file + the Associated Domains capability in Xcode) -- iOS intercepts Universal Links at the OS level before any browser loads them, so restrictive mail-app browsers can't block the handoff. Needs a domain (none currently configured for this beyond the in-app marketing page) -- confirm with user whether one exists/should be acquired. (2) Edit Authentication &gt; Email Templates &gt; Magic Link in the Supabase dashboard: change subject + body copy to say 'Shema', give the link friendly anchor text ('Open in Shema') instead of a bare URL. Also flagged: Supabase's default built-in email sender has a low rate limit (dev/testing tier) -- worth Custom SMTP (Resend/Postmark/etc.) before many pastors test magic-link sign-in around the same time, which fixes branding AND the rate limit together.</t>
-        </is>
-      </c>
-      <c r="H87" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>PARKED -- needs a domain, which the user doesn't have yet (decided 2026-07-23). The robust fix is a Universal Link (a real https:// URL on a domain we control, with an apple-app-site-association file + Xcode's Associated Domains capability) instead of the com.shema.app:// custom scheme -- iOS intercepts Universal Links at the OS level before any browser loads them, so a restrictive mail-app in-app browser can't block the handoff the way it currently does. Revisit once a domain exists (could piggyback on whatever domain ends up hosting marketing/support, if one is ever set up).</t>
+        </is>
+      </c>
+      <c r="H87" s="24" t="inlineStr">
+        <is>
+          <t>Parked</t>
         </is>
       </c>
       <c r="I87" s="8" t="inlineStr">
@@ -4851,7 +4854,57 @@
       </c>
       <c r="J87" s="8" t="inlineStr">
         <is>
-          <t>Recommend for the beta: tell pastors to use Continue with Google if possible (fully working), or open magic-link emails via 'Open in Safari' if they hit this. Full Universal Links fix and/or Custom SMTP are real but non-trivial follow-ups -- scope with user before building.</t>
+          <t>Interim guidance for the beta stands: lead pastors to 'Continue with Google' (fully working); if anyone uses the magic link, tell them to 'Open in Safari' rather than tapping it inside their mail app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="140" customHeight="1">
+      <c r="A88" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Account/Auth</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Magic-link email shows no Shema branding -- raw Supabase URL only</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>Split out of #83 (device report): the sign-in email itself has no Shema name/styling, just a bare Supabase project link as the visible text.</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>Supabase's built-in Auth email templates are unbranded by default -- the Magic Link template just wraps the raw {{ .ConfirmationURL }} link with no styling or copy.</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>Dashboard-only fix (not app code): replace the Magic Link template's subject + HTML body in Supabase Dashboard &gt; Authentication &gt; Email Templates &gt; Magic Link with Shema-branded copy (cream/forest/gold palette matching the app, 'Open in Shema' button instead of a bare link). Exact paste-in subject + HTML handed to the user in chat 2026-07-23. Does not touch the underlying link mechanism -- #83's return-to-app issue is separate and still applies until Universal Links exist.</t>
+        </is>
+      </c>
+      <c r="H88" s="12" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>Awaiting user: paste the provided template into the Supabase dashboard, send a test magic link, confirm it now shows Shema branding.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ProPresenter export overhaul: rename toggle, drop auto title/headers, slide-break splitting, match Present styling
Renames the per-item export toggle "Slide" -> "Screen". exportForProPresenter()
no longer injects the sermon title or section headers -- it exports exactly the
items toggled on, with scripture defaulting on and everything else defaulting
off. Adds a manual slide-break marker (new scissors button in the rich-text
toolbar) so one scripture item can span multiple ProPresenter slides without
splitting Prepare/Present's view of the passage. RTF styling now mirrors
Present's own per-type look (gold italic serif for scripture, orange italic
serif for illustrations, muted italic for quiet asides) instead of plain
black Calibri.

Ticket #85.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -627,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4905,6 +4905,56 @@
       <c r="J88" s="5" t="inlineStr">
         <is>
           <t>Awaiting user: paste the provided template into the Supabase dashboard, send a test magic link, confirm it now shows Shema branding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>85</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>ProPresenter Export</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>ProPresenter export overhaul: rename toggle, drop auto title/headers, slide-break splitting, match Present styling</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>User feedback on the ProPresenter export/toggle: (1) the per-item toggle labeled "Slide" wasn't intuitive -- every item already looks like a slide once you hit Present. (2) The export auto-added the sermon title and each section header as its own slide, which the user did not want -- only what the pastor actually selects should export (scripture excepted, still on by default). (3) A long scripture passage pasted as one item became one wall-of-text ProPresenter slide, with no way to split it -- asked for a graceful way to break it up, open to changing how scripture is added in Prepare if needed. (4) Wanted the exported .rtf to visually match Present (font, color) instead of reading like a plain black-Calibri afterthought.</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>All four were real gaps in the original #65 ProPresenter export: (1) naming didn't distinguish "shown in Present" from "pushed to the venue screen." (2) exportForProPresenter() unconditionally injected the sermon title + each section title as their own RTF slides on top of whatever items were toggled on. (3) one item = one RTF paragraph with no way to subdivide it, so a multi-verse passage in a single item became a single slide regardless of length. (4) the RTF only highlighted inline scripture citations in blue -- it never carried Present's own per-type styling (.line.scripture / .line.illustration / .line.quiet) into the export.</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Renamed the toggle "Slide" -&gt; "Screen" (button + title text). Rewrote exportForProPresenter() to flatten toggled items straight into RTF paragraphs with no sermon-title or section-header slides ever injected; proIncluded() default narrowed to scripture-only (illustrations and everything else now need an explicit tap, matching "just what the user selects"). Added a new slide-break marker (.pp-break, makeSlideBreakMarkerHtml/splitItemHtmlOnBreaks) inserted via a new scissors button in the rich-text toolbar (#slideBreakBtn) -- a pastor drops it mid-passage in any item's own text; Present/Practice keep rendering that item as one continuous flowing block (marker is display:none on stage), while the export cuts to a new RTF paragraph/slide at each marker. sanitizeRichText special-cases the marker (preserved verbatim, like the Import stage's own .import-break); htmlToPlainText strips it everywhere else (search, manuscript) so it never leaks into text; a new stripSlideBreaks() removes just the marker from the manuscript export while keeping real formatting intact. RTF styling now mirrors Present per type: scripture = gold italic Georgia (serif), illustration = orange italic Georgia, quiet = muted italic, block = plain -- new f1 Georgia font-table entry and cf2-4 color-table entries; the old blue inline-citation highlight moved to its own cf5 so it no longer collides with a scripture item's own gold styling.</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Verified end-to-end with Playwright (serviceWorkers:"block" on the browser context avoids a harness-specific issue where the real sw.js install fetch was silently re-fetching vendor/purchases-capacitor.js and clobbering the Capacitor mock): toggle reads "Screen"; scripture defaults on, block/illustration default off; toggling illustration on includes it styled orange/italic/Georgia; export has zero sermon-title/section-header text; scissors button in the real toolbar inserts a real .pp-break marker and the brk-del "x" removes it; a marked scripture item splits into two separate RTF slide paragraphs; Present hides the marker (display:none) and still renders the passage as one block; the manuscript export keeps both verse chunks and drops the marker text. Bumped sw.js v98 -&gt; v99.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix literal &nbsp; leaking into ProPresenter export after slide breaks
A tag-free scripture chunk (common right at a slide-break boundary) was
getting misread as legacy plain text by htmlToPlainText's ambiguity
heuristic and double-escaped, turning a real non-breaking-space entity into
literal visible "&nbsp;" text on the exported slide. Added
richHtmlToPlainText() for per-chunk conversion (always parses as HTML, no
ambiguity) and normalize an item's text through the same
sanitizeRichText(seedRichHtml(...)) pipeline every other consumer uses
before splitting it on breaks.

Ticket #85.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -656,6 +656,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4939,7 +4940,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Renamed the toggle "Slide" -&gt; "Screen" (button + title text). Rewrote exportForProPresenter() to flatten toggled items straight into RTF paragraphs with no sermon-title or section-header slides ever injected; proIncluded() default narrowed to scripture-only (illustrations and everything else now need an explicit tap, matching "just what the user selects"). Added a new slide-break marker (.pp-break, makeSlideBreakMarkerHtml/splitItemHtmlOnBreaks) inserted via a new scissors button in the rich-text toolbar (#slideBreakBtn) -- a pastor drops it mid-passage in any item's own text; Present/Practice keep rendering that item as one continuous flowing block (marker is display:none on stage), while the export cuts to a new RTF paragraph/slide at each marker. sanitizeRichText special-cases the marker (preserved verbatim, like the Import stage's own .import-break); htmlToPlainText strips it everywhere else (search, manuscript) so it never leaks into text; a new stripSlideBreaks() removes just the marker from the manuscript export while keeping real formatting intact. RTF styling now mirrors Present per type: scripture = gold italic Georgia (serif), illustration = orange italic Georgia, quiet = muted italic, block = plain -- new f1 Georgia font-table entry and cf2-4 color-table entries; the old blue inline-citation highlight moved to its own cf5 so it no longer collides with a scripture item's own gold styling.</t>
+          <t>Renamed the toggle "Slide" -&gt; "Screen" (button + title text). Rewrote exportForProPresenter() to flatten toggled items straight into RTF paragraphs with no sermon-title or section-header slides ever injected; proIncluded() default narrowed to scripture-only (illustrations and everything else now need an explicit tap, matching "just what the user selects"). Added a new slide-break marker (.pp-break, makeSlideBreakMarkerHtml/splitItemHtmlOnBreaks) inserted via a new scissors button in the rich-text toolbar (#slideBreakBtn) -- a pastor drops it mid-passage in any item's own text; Present/Practice keep rendering that item as one continuous flowing block (marker is display:none on stage), while the export cuts to a new RTF paragraph/slide at each marker. sanitizeRichText special-cases the marker (preserved verbatim, like the Import stage's own .import-break); htmlToPlainText strips it everywhere else (search, manuscript) so it never leaks into text; a new stripSlideBreaks() removes just the marker from the manuscript export while keeping real formatting intact. RTF styling now mirrors Present per type: scripture = gold italic Georgia (serif), illustration = orange italic Georgia, quiet = muted italic, block = plain -- new f1 Georgia font-table entry and cf2-4 color-table entries; the old blue inline-citation highlight moved to its own cf5 so it no longer collides with a scripture item's own gold styling. FOLLOW-UP FIX (device report): a scripture chunk with a literal non-breaking-space character (common at the end of a Word/BLB-pasted verse) and no other tags was getting double-escaped -- htmlToPlainText's legacy-plain-text-vs-rich-HTML heuristic (checks for the presence of "&lt;") misclassified a tag-free HTML fragment as legacy text and ran it through escapeHtml() a second time, turning the real &amp;nbsp; entity into literal visible "&amp;nbsp;" text on the slide. Added richHtmlToPlainText() (always parses as HTML, no legacy-detection ambiguity) for the per-chunk conversion, and rtfParagraphsForItem now normalizes an item's text via sanitizeRichText(seedRichHtml(...)) -- same as every other consumer -- before splitting it, so a chunk is always guaranteed-real HTML.</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -4949,12 +4950,12 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>Needs Testing</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Verified end-to-end with Playwright (serviceWorkers:"block" on the browser context avoids a harness-specific issue where the real sw.js install fetch was silently re-fetching vendor/purchases-capacitor.js and clobbering the Capacitor mock): toggle reads "Screen"; scripture defaults on, block/illustration default off; toggling illustration on includes it styled orange/italic/Georgia; export has zero sermon-title/section-header text; scissors button in the real toolbar inserts a real .pp-break marker and the brk-del "x" removes it; a marked scripture item splits into two separate RTF slide paragraphs; Present hides the marker (display:none) and still renders the passage as one block; the manuscript export keeps both verse chunks and drops the marker text. Bumped sw.js v98 -&gt; v99.</t>
+          <t>Verified end-to-end with Playwright (serviceWorkers:"block" on the browser context avoids a harness-specific issue where the real sw.js install fetch was silently re-fetching vendor/purchases-capacitor.js and clobbering the Capacitor mock): toggle reads "Screen"; scripture defaults on, block/illustration default off; toggling illustration on includes it styled orange/italic/Georgia; export has zero sermon-title/section-header text; scissors button in the real toolbar inserts a real .pp-break marker and the brk-del "x" removes it; a marked scripture item splits into two separate RTF slide paragraphs; Present hides the marker (display:none) and still renders the passage as one block; the manuscript export keeps both verse chunks and drops the marker text. Bumped sw.js v98 -&gt; v99. UPDATE: device test surfaced the &amp;nbsp; bug above (fixed, bumped sw.js v99-&gt;v100) plus a bigger finding -- ProPresenter's own RTF/Word import only preserves formatting that varies WITHIN a text box (e.g. one bolded/colored word among plain text); it discards formatting that's uniform across an entire slide's text and falls back to the slide's theme default instead (confirmed via Renewed Vision's own support docs). Since our per-type styling colors/italicizes an ENTIRE scripture/illustration body uniformly, ProPresenter is very likely discarding it on import regardless of what our RTF says -- this looks like the real explanation for "none of this retained the formatting" in the device screenshot, not an RTF-syntax bug. Flagged to the user for a decision on how to proceed; the inline scripture-citation highlight (a citation mentioned inline within otherwise-plain prose) is unaffected since THAT varies within the box and should still survive import.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop whole-body RTF styling from ProPresenter export
ProPresenter's RTF/Word import only keeps formatting that varies within a
text box; it discards formatting that's uniform across an entire slide and
falls back to that slide's theme instead. The per-type gold/orange italic
styling added earlier was invisible after a real import. Reverted the
export back to plain text, keeping only the inline scripture-citation
highlight (which does vary within a box). Matching Present's look is left
to a ProPresenter Theme set up in ProPresenter itself.

Ticket #85.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -4940,7 +4940,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Renamed the toggle "Slide" -&gt; "Screen" (button + title text). Rewrote exportForProPresenter() to flatten toggled items straight into RTF paragraphs with no sermon-title or section-header slides ever injected; proIncluded() default narrowed to scripture-only (illustrations and everything else now need an explicit tap, matching "just what the user selects"). Added a new slide-break marker (.pp-break, makeSlideBreakMarkerHtml/splitItemHtmlOnBreaks) inserted via a new scissors button in the rich-text toolbar (#slideBreakBtn) -- a pastor drops it mid-passage in any item's own text; Present/Practice keep rendering that item as one continuous flowing block (marker is display:none on stage), while the export cuts to a new RTF paragraph/slide at each marker. sanitizeRichText special-cases the marker (preserved verbatim, like the Import stage's own .import-break); htmlToPlainText strips it everywhere else (search, manuscript) so it never leaks into text; a new stripSlideBreaks() removes just the marker from the manuscript export while keeping real formatting intact. RTF styling now mirrors Present per type: scripture = gold italic Georgia (serif), illustration = orange italic Georgia, quiet = muted italic, block = plain -- new f1 Georgia font-table entry and cf2-4 color-table entries; the old blue inline-citation highlight moved to its own cf5 so it no longer collides with a scripture item's own gold styling. FOLLOW-UP FIX (device report): a scripture chunk with a literal non-breaking-space character (common at the end of a Word/BLB-pasted verse) and no other tags was getting double-escaped -- htmlToPlainText's legacy-plain-text-vs-rich-HTML heuristic (checks for the presence of "&lt;") misclassified a tag-free HTML fragment as legacy text and ran it through escapeHtml() a second time, turning the real &amp;nbsp; entity into literal visible "&amp;nbsp;" text on the slide. Added richHtmlToPlainText() (always parses as HTML, no legacy-detection ambiguity) for the per-chunk conversion, and rtfParagraphsForItem now normalizes an item's text via sanitizeRichText(seedRichHtml(...)) -- same as every other consumer -- before splitting it, so a chunk is always guaranteed-real HTML.</t>
+          <t>Renamed the toggle "Slide" -&gt; "Screen" (button + title text). Rewrote exportForProPresenter() to flatten toggled items straight into RTF paragraphs with no sermon-title or section-header slides ever injected; proIncluded() default narrowed to scripture-only (illustrations and everything else now need an explicit tap, matching "just what the user selects"). Added a new slide-break marker (.pp-break, makeSlideBreakMarkerHtml/splitItemHtmlOnBreaks) inserted via a new scissors button in the rich-text toolbar (#slideBreakBtn) -- a pastor drops it mid-passage in any item's own text; Present/Practice keep rendering that item as one continuous flowing block (marker is display:none on stage), while the export cuts to a new RTF paragraph/slide at each marker. sanitizeRichText special-cases the marker (preserved verbatim, like the Import stage's own .import-break); htmlToPlainText strips it everywhere else (search, manuscript) so it never leaks into text; a new stripSlideBreaks() removes just the marker from the manuscript export while keeping real formatting intact. RTF styling now mirrors Present per type: scripture = gold italic Georgia (serif), illustration = orange italic Georgia, quiet = muted italic, block = plain -- new f1 Georgia font-table entry and cf2-4 color-table entries; the old blue inline-citation highlight moved to its own cf5 so it no longer collides with a scripture item's own gold styling. FOLLOW-UP FIX (device report): a scripture chunk with a literal non-breaking-space character (common at the end of a Word/BLB-pasted verse) and no other tags was getting double-escaped -- htmlToPlainText's legacy-plain-text-vs-rich-HTML heuristic (checks for the presence of "&lt;") misclassified a tag-free HTML fragment as legacy text and ran it through escapeHtml() a second time, turning the real &amp;nbsp; entity into literal visible "&amp;nbsp;" text on the slide. Added richHtmlToPlainText() (always parses as HTML, no legacy-detection ambiguity) for the per-chunk conversion, and rtfParagraphsForItem now normalizes an item's text via sanitizeRichText(seedRichHtml(...)) -- same as every other consumer -- before splitting it, so a chunk is always guaranteed-real HTML. DECIDED (2026-07-27): dropped the whole-body per-type styling entirely per user choice -- reverted the export back to plain text (font table back to just Calibri, color table back to just ink + the one blue inline-citation highlight). Matching Present visually is left to a ProPresenter Theme set up once inside ProPresenter itself.</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -4955,7 +4955,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Verified end-to-end with Playwright (serviceWorkers:"block" on the browser context avoids a harness-specific issue where the real sw.js install fetch was silently re-fetching vendor/purchases-capacitor.js and clobbering the Capacitor mock): toggle reads "Screen"; scripture defaults on, block/illustration default off; toggling illustration on includes it styled orange/italic/Georgia; export has zero sermon-title/section-header text; scissors button in the real toolbar inserts a real .pp-break marker and the brk-del "x" removes it; a marked scripture item splits into two separate RTF slide paragraphs; Present hides the marker (display:none) and still renders the passage as one block; the manuscript export keeps both verse chunks and drops the marker text. Bumped sw.js v98 -&gt; v99. UPDATE: device test surfaced the &amp;nbsp; bug above (fixed, bumped sw.js v99-&gt;v100) plus a bigger finding -- ProPresenter's own RTF/Word import only preserves formatting that varies WITHIN a text box (e.g. one bolded/colored word among plain text); it discards formatting that's uniform across an entire slide's text and falls back to the slide's theme default instead (confirmed via Renewed Vision's own support docs). Since our per-type styling colors/italicizes an ENTIRE scripture/illustration body uniformly, ProPresenter is very likely discarding it on import regardless of what our RTF says -- this looks like the real explanation for "none of this retained the formatting" in the device screenshot, not an RTF-syntax bug. Flagged to the user for a decision on how to proceed; the inline scripture-citation highlight (a citation mentioned inline within otherwise-plain prose) is unaffected since THAT varies within the box and should still survive import.</t>
+          <t>Verified end-to-end with Playwright (serviceWorkers:"block" on the browser context avoids a harness-specific issue where the real sw.js install fetch was silently re-fetching vendor/purchases-capacitor.js and clobbering the Capacitor mock): toggle reads "Screen"; scripture defaults on, block/illustration default off; toggling illustration on includes it styled orange/italic/Georgia; export has zero sermon-title/section-header text; scissors button in the real toolbar inserts a real .pp-break marker and the brk-del "x" removes it; a marked scripture item splits into two separate RTF slide paragraphs; Present hides the marker (display:none) and still renders the passage as one block; the manuscript export keeps both verse chunks and drops the marker text. Bumped sw.js v98 -&gt; v99. UPDATE: device test surfaced the &amp;nbsp; bug above (fixed, bumped sw.js v99-&gt;v100) plus a bigger finding -- ProPresenter's own RTF/Word import only preserves formatting that varies WITHIN a text box (e.g. one bolded/colored word among plain text); it discards formatting that's uniform across an entire slide's text and falls back to the slide's theme default instead (confirmed via Renewed Vision's own support docs). Since our per-type styling colors/italicizes an ENTIRE scripture/illustration body uniformly, ProPresenter is very likely discarding it on import regardless of what our RTF says -- this looks like the real explanation for "none of this retained the formatting" in the device screenshot, not an RTF-syntax bug. Flagged to the user for a decision on how to proceed; the inline scripture-citation highlight (a citation mentioned inline within otherwise-plain prose) is unaffected since THAT varies within the box and should still survive import. User chose "drop it, keep export plain" over keeping the inert styling. Re-verified with Playwright: export is plain text again, &amp;nbsp; fix still holds, slide-break splitting still works, toggle defaults unchanged. Bumped sw.js v100-&gt;v101. Awaiting a real ProPresenter import test to confirm the &amp;nbsp; artifact is gone and slides read as expected now.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Strip page chrome (buttons, icons) from pasted Bible-lookup-site content
Pasting a verse directly off a Bible-lookup website into a scripture item
carried that page's own per-verse "Tools" button and copy icon along as
literal text, since item text fields had no paste handler and the
sanitizer unwrapped disallowed tags while keeping their content -- correct
for a stray formatting div, wrong for chrome whose label text isn't sermon
content. sanitizeRichText and the Import stage's sanitizeImportHtml now
both hard-drop BUTTON/INPUT/SELECT/TEXTAREA/SVG/NAV/NOSCRIPT and
role="button" elements outright, and item text fields sanitize clipboard
HTML before insertion instead of after.

Ticket #85.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -4940,7 +4940,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Renamed the toggle "Slide" -&gt; "Screen" (button + title text). Rewrote exportForProPresenter() to flatten toggled items straight into RTF paragraphs with no sermon-title or section-header slides ever injected; proIncluded() default narrowed to scripture-only (illustrations and everything else now need an explicit tap, matching "just what the user selects"). Added a new slide-break marker (.pp-break, makeSlideBreakMarkerHtml/splitItemHtmlOnBreaks) inserted via a new scissors button in the rich-text toolbar (#slideBreakBtn) -- a pastor drops it mid-passage in any item's own text; Present/Practice keep rendering that item as one continuous flowing block (marker is display:none on stage), while the export cuts to a new RTF paragraph/slide at each marker. sanitizeRichText special-cases the marker (preserved verbatim, like the Import stage's own .import-break); htmlToPlainText strips it everywhere else (search, manuscript) so it never leaks into text; a new stripSlideBreaks() removes just the marker from the manuscript export while keeping real formatting intact. RTF styling now mirrors Present per type: scripture = gold italic Georgia (serif), illustration = orange italic Georgia, quiet = muted italic, block = plain -- new f1 Georgia font-table entry and cf2-4 color-table entries; the old blue inline-citation highlight moved to its own cf5 so it no longer collides with a scripture item's own gold styling. FOLLOW-UP FIX (device report): a scripture chunk with a literal non-breaking-space character (common at the end of a Word/BLB-pasted verse) and no other tags was getting double-escaped -- htmlToPlainText's legacy-plain-text-vs-rich-HTML heuristic (checks for the presence of "&lt;") misclassified a tag-free HTML fragment as legacy text and ran it through escapeHtml() a second time, turning the real &amp;nbsp; entity into literal visible "&amp;nbsp;" text on the slide. Added richHtmlToPlainText() (always parses as HTML, no legacy-detection ambiguity) for the per-chunk conversion, and rtfParagraphsForItem now normalizes an item's text via sanitizeRichText(seedRichHtml(...)) -- same as every other consumer -- before splitting it, so a chunk is always guaranteed-real HTML. DECIDED (2026-07-27): dropped the whole-body per-type styling entirely per user choice -- reverted the export back to plain text (font table back to just Calibri, color table back to just ink + the one blue inline-citation highlight). Matching Present visually is left to a ProPresenter Theme set up once inside ProPresenter itself.</t>
+          <t>Renamed the toggle "Slide" -&gt; "Screen" (button + title text). Rewrote exportForProPresenter() to flatten toggled items straight into RTF paragraphs with no sermon-title or section-header slides ever injected; proIncluded() default narrowed to scripture-only (illustrations and everything else now need an explicit tap, matching "just what the user selects"). Added a new slide-break marker (.pp-break, makeSlideBreakMarkerHtml/splitItemHtmlOnBreaks) inserted via a new scissors button in the rich-text toolbar (#slideBreakBtn) -- a pastor drops it mid-passage in any item's own text; Present/Practice keep rendering that item as one continuous flowing block (marker is display:none on stage), while the export cuts to a new RTF paragraph/slide at each marker. sanitizeRichText special-cases the marker (preserved verbatim, like the Import stage's own .import-break); htmlToPlainText strips it everywhere else (search, manuscript) so it never leaks into text; a new stripSlideBreaks() removes just the marker from the manuscript export while keeping real formatting intact. RTF styling now mirrors Present per type: scripture = gold italic Georgia (serif), illustration = orange italic Georgia, quiet = muted italic, block = plain -- new f1 Georgia font-table entry and cf2-4 color-table entries; the old blue inline-citation highlight moved to its own cf5 so it no longer collides with a scripture item's own gold styling. FOLLOW-UP FIX (device report): a scripture chunk with a literal non-breaking-space character (common at the end of a Word/BLB-pasted verse) and no other tags was getting double-escaped -- htmlToPlainText's legacy-plain-text-vs-rich-HTML heuristic (checks for the presence of "&lt;") misclassified a tag-free HTML fragment as legacy text and ran it through escapeHtml() a second time, turning the real &amp;nbsp; entity into literal visible "&amp;nbsp;" text on the slide. Added richHtmlToPlainText() (always parses as HTML, no legacy-detection ambiguity) for the per-chunk conversion, and rtfParagraphsForItem now normalizes an item's text via sanitizeRichText(seedRichHtml(...)) -- same as every other consumer -- before splitting it, so a chunk is always guaranteed-real HTML. DECIDED (2026-07-27): dropped the whole-body per-type styling entirely per user choice -- reverted the export back to plain text (font table back to just Calibri, color table back to just ink + the one blue inline-citation highlight). Matching Present visually is left to a ProPresenter Theme set up once inside ProPresenter itself. FURTHER FIX (device report): pasting a verse straight off a Bible-lookup website (Blue Letter Bible) into a scripture item brought along that page's own per-verse "Tools" button and copy-icon chrome as literal text/elements, because the item text field had no paste handler of its own -- the browser inserted the raw pasted HTML directly into the editor, and the existing sanitizer (sanitizeRichText) UNWRAPPED disallowed tags (like &lt;button&gt;) while keeping their text content, which is correct for a stray formatting &lt;div&gt;/&lt;span&gt; but wrong for page chrome whose label text isn't sermon content. Fixed two ways: (1) sanitizeRichText and the Import stage's sanitizeImportHtml both now hard-drop BUTTON/INPUT/SELECT/TEXTAREA/SVG/NAV/NOSCRIPT and role=button elements entirely (tag AND content removed) instead of unwrapping them, via a shared isChromeElement() check. (2) Added a dedicated 'paste' handler on item text fields (mirroring the Import stage's own paste handler) that sanitizes clipboard HTML BEFORE insertion, so chrome never touches the live editor DOM in the first place -- previously it relied on the browser's raw paste + sanitize-on-next-input, which left visible buttons sitting in the editor until the item happened to re-render.</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -4955,7 +4955,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Verified end-to-end with Playwright (serviceWorkers:"block" on the browser context avoids a harness-specific issue where the real sw.js install fetch was silently re-fetching vendor/purchases-capacitor.js and clobbering the Capacitor mock): toggle reads "Screen"; scripture defaults on, block/illustration default off; toggling illustration on includes it styled orange/italic/Georgia; export has zero sermon-title/section-header text; scissors button in the real toolbar inserts a real .pp-break marker and the brk-del "x" removes it; a marked scripture item splits into two separate RTF slide paragraphs; Present hides the marker (display:none) and still renders the passage as one block; the manuscript export keeps both verse chunks and drops the marker text. Bumped sw.js v98 -&gt; v99. UPDATE: device test surfaced the &amp;nbsp; bug above (fixed, bumped sw.js v99-&gt;v100) plus a bigger finding -- ProPresenter's own RTF/Word import only preserves formatting that varies WITHIN a text box (e.g. one bolded/colored word among plain text); it discards formatting that's uniform across an entire slide's text and falls back to the slide's theme default instead (confirmed via Renewed Vision's own support docs). Since our per-type styling colors/italicizes an ENTIRE scripture/illustration body uniformly, ProPresenter is very likely discarding it on import regardless of what our RTF says -- this looks like the real explanation for "none of this retained the formatting" in the device screenshot, not an RTF-syntax bug. Flagged to the user for a decision on how to proceed; the inline scripture-citation highlight (a citation mentioned inline within otherwise-plain prose) is unaffected since THAT varies within the box and should still survive import. User chose "drop it, keep export plain" over keeping the inert styling. Re-verified with Playwright: export is plain text again, &amp;nbsp; fix still holds, slide-break splitting still works, toggle defaults unchanged. Bumped sw.js v100-&gt;v101. Awaiting a real ProPresenter import test to confirm the &amp;nbsp; artifact is gone and slides read as expected now.</t>
+          <t>Verified end-to-end with Playwright (serviceWorkers:"block" on the browser context avoids a harness-specific issue where the real sw.js install fetch was silently re-fetching vendor/purchases-capacitor.js and clobbering the Capacitor mock): toggle reads "Screen"; scripture defaults on, block/illustration default off; toggling illustration on includes it styled orange/italic/Georgia; export has zero sermon-title/section-header text; scissors button in the real toolbar inserts a real .pp-break marker and the brk-del "x" removes it; a marked scripture item splits into two separate RTF slide paragraphs; Present hides the marker (display:none) and still renders the passage as one block; the manuscript export keeps both verse chunks and drops the marker text. Bumped sw.js v98 -&gt; v99. UPDATE: device test surfaced the &amp;nbsp; bug above (fixed, bumped sw.js v99-&gt;v100) plus a bigger finding -- ProPresenter's own RTF/Word import only preserves formatting that varies WITHIN a text box (e.g. one bolded/colored word among plain text); it discards formatting that's uniform across an entire slide's text and falls back to the slide's theme default instead (confirmed via Renewed Vision's own support docs). Since our per-type styling colors/italicizes an ENTIRE scripture/illustration body uniformly, ProPresenter is very likely discarding it on import regardless of what our RTF says -- this looks like the real explanation for "none of this retained the formatting" in the device screenshot, not an RTF-syntax bug. Flagged to the user for a decision on how to proceed; the inline scripture-citation highlight (a citation mentioned inline within otherwise-plain prose) is unaffected since THAT varies within the box and should still survive import. User chose "drop it, keep export plain" over keeping the inert styling. Re-verified with Playwright: export is plain text again, &amp;nbsp; fix still holds, slide-break splitting still works, toggle defaults unchanged. Bumped sw.js v100-&gt;v101. Awaiting a real ProPresenter import test to confirm the &amp;nbsp; artifact is gone and slides read as expected now. Re-verified with Playwright (21 checks): simulated a clipboard paste with &lt;button&gt;Tools&lt;/button&gt; and &lt;svg&gt; icons mixed into real verse text -- button text and svg both stripped, verse references and body text both survive intact; all prior checks (toggle defaults, no title/headers, nbsp fix, slide-break splitting, plain export) still pass. Bumped sw.js v101-&gt;v102. NOTE: this session runs in a fresh container that started from an older commit than the branch's actual HEAD -- had to fast-forward-merge to origin/claude/app-store-paid-launch-1jkhur before continuing, since the previous 3 commits (nbsp fix, style revert) existed on the remote but not in this container's local checkout.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Highlight button to the Import Notes toolbar
Mirrors the Prepare item editor's own highlight button: wraps the current
selection in a bare <mark> via the Range API (not a real execCommand), or
unwraps it if the selection already sits inside one. IMPORT_ALLOWED_TAGS
already keeps MARK through the paste/upload sanitizer and the
section-split, so a highlighted quote survives into the resulting Prepare
item untouched.

Ticket #87. Also logs #86 (Parked) to revisit the Bible-lookup-site
paste-sanitizer's robustness later, and marks #85 Done per user
confirmation.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -627,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J89"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -656,7 +656,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4950,12 +4949,112 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Needs Testing</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Verified end-to-end with Playwright (serviceWorkers:"block" on the browser context avoids a harness-specific issue where the real sw.js install fetch was silently re-fetching vendor/purchases-capacitor.js and clobbering the Capacitor mock): toggle reads "Screen"; scripture defaults on, block/illustration default off; toggling illustration on includes it styled orange/italic/Georgia; export has zero sermon-title/section-header text; scissors button in the real toolbar inserts a real .pp-break marker and the brk-del "x" removes it; a marked scripture item splits into two separate RTF slide paragraphs; Present hides the marker (display:none) and still renders the passage as one block; the manuscript export keeps both verse chunks and drops the marker text. Bumped sw.js v98 -&gt; v99. UPDATE: device test surfaced the &amp;nbsp; bug above (fixed, bumped sw.js v99-&gt;v100) plus a bigger finding -- ProPresenter's own RTF/Word import only preserves formatting that varies WITHIN a text box (e.g. one bolded/colored word among plain text); it discards formatting that's uniform across an entire slide's text and falls back to the slide's theme default instead (confirmed via Renewed Vision's own support docs). Since our per-type styling colors/italicizes an ENTIRE scripture/illustration body uniformly, ProPresenter is very likely discarding it on import regardless of what our RTF says -- this looks like the real explanation for "none of this retained the formatting" in the device screenshot, not an RTF-syntax bug. Flagged to the user for a decision on how to proceed; the inline scripture-citation highlight (a citation mentioned inline within otherwise-plain prose) is unaffected since THAT varies within the box and should still survive import. User chose "drop it, keep export plain" over keeping the inert styling. Re-verified with Playwright: export is plain text again, &amp;nbsp; fix still holds, slide-break splitting still works, toggle defaults unchanged. Bumped sw.js v100-&gt;v101. Awaiting a real ProPresenter import test to confirm the &amp;nbsp; artifact is gone and slides read as expected now. Re-verified with Playwright (21 checks): simulated a clipboard paste with &lt;button&gt;Tools&lt;/button&gt; and &lt;svg&gt; icons mixed into real verse text -- button text and svg both stripped, verse references and body text both survive intact; all prior checks (toggle defaults, no title/headers, nbsp fix, slide-break splitting, plain export) still pass. Bumped sw.js v101-&gt;v102. NOTE: this session runs in a fresh container that started from an older commit than the branch's actual HEAD -- had to fast-forward-merge to origin/claude/app-store-paid-launch-1jkhur before continuing, since the previous 3 commits (nbsp fix, style revert) existed on the remote but not in this container's local checkout.</t>
+          <t>Verified end-to-end with Playwright (serviceWorkers:"block" on the browser context avoids a harness-specific issue where the real sw.js install fetch was silently re-fetching vendor/purchases-capacitor.js and clobbering the Capacitor mock): toggle reads "Screen"; scripture defaults on, block/illustration default off; toggling illustration on includes it styled orange/italic/Georgia; export has zero sermon-title/section-header text; scissors button in the real toolbar inserts a real .pp-break marker and the brk-del "x" removes it; a marked scripture item splits into two separate RTF slide paragraphs; Present hides the marker (display:none) and still renders the passage as one block; the manuscript export keeps both verse chunks and drops the marker text. Bumped sw.js v98 -&gt; v99. UPDATE: device test surfaced the &amp;nbsp; bug above (fixed, bumped sw.js v99-&gt;v100) plus a bigger finding -- ProPresenter's own RTF/Word import only preserves formatting that varies WITHIN a text box (e.g. one bolded/colored word among plain text); it discards formatting that's uniform across an entire slide's text and falls back to the slide's theme default instead (confirmed via Renewed Vision's own support docs). Since our per-type styling colors/italicizes an ENTIRE scripture/illustration body uniformly, ProPresenter is very likely discarding it on import regardless of what our RTF says -- this looks like the real explanation for "none of this retained the formatting" in the device screenshot, not an RTF-syntax bug. Flagged to the user for a decision on how to proceed; the inline scripture-citation highlight (a citation mentioned inline within otherwise-plain prose) is unaffected since THAT varies within the box and should still survive import. User chose "drop it, keep export plain" over keeping the inert styling. Re-verified with Playwright: export is plain text again, &amp;nbsp; fix still holds, slide-break splitting still works, toggle defaults unchanged. Bumped sw.js v100-&gt;v101. Awaiting a real ProPresenter import test to confirm the &amp;nbsp; artifact is gone and slides read as expected now. Re-verified with Playwright (21 checks): simulated a clipboard paste with &lt;button&gt;Tools&lt;/button&gt; and &lt;svg&gt; icons mixed into real verse text -- button text and svg both stripped, verse references and body text both survive intact; all prior checks (toggle defaults, no title/headers, nbsp fix, slide-break splitting, plain export) still pass. Bumped sw.js v101-&gt;v102. NOTE: this session runs in a fresh container that started from an older commit than the branch's actual HEAD -- had to fast-forward-merge to origin/claude/app-store-paid-launch-1jkhur before continuing, since the previous 3 commits (nbsp fix, style revert) existed on the remote but not in this container's local checkout. User confirmed (2026-07-27) it is functioning for now. Split the paste-sanitizer robustness question out to #86 (Parked) rather than leave it open-ended on this ticket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>86</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Prepare/Editor</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Revisit paste-sanitizer robustness for Bible-lookup-site content</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Follow-up from #85: the tag-based drop list (BUTTON/INPUT/SELECT/TEXTAREA/SVG/NAV/NOSCRIPT + role=button) fixed the specific Blue Letter Bible "Tools" button/icon case, but user flagged wanting to revisit this later rather than treat it as fully solved.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>The current fix is an allowlist/denylist heuristic on raw pasted HTML -- robust against the sites tested so far, but any Bible-lookup or note-taking site with different chrome markup (a styled &lt;a&gt;/&lt;div role=button&gt;-alike element we have not seen, a differently-structured verse-reference widget, etc.) could still leak stray UI text the same way, since the sanitizer cannot know every site's markup in advance.</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>PARKED -- not actioned. Possible directions to consider later: (1) a dedicated, purpose-built scripture paste/lookup flow (referenced but deferred in #78/#79) instead of relying on generic clipboard sanitization of arbitrary webpages; (2) a more aggressive heuristic (e.g. treat any element whose own direct text is short and matches known chrome vocabulary like "Tools"/"Copy"/"Share" as chrome regardless of tag); (3) simply keep monitoring for further device reports and extend the drop-list reactively as real sites surface new cases.</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Parked</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>User: "Make a note to revisit this later, I think it is functioning for now." Logged as its own ticket so #85 (now Done) does not stay open-ended.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>87</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Add Highlight button to the Import Notes toolbar</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>User request: add the same highlight (yellow &lt;mark&gt;) capability the Prepare item editor already has to the Import tool's own toolbar, so a pastor can mark up an important quote/phrase while staging pasted notes, before they are split into sections.</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Added #importHighlightBtn to #importToolbar (after Underline), styled to match the existing #highlightBtn. Wired with the same manual Range-API approach as the Prepare editor's highlight button (highlight is not a real execCommand): wraps the current selection in a bare &lt;mark&gt;, or unwraps it if the selection already sits inside one, reusing the existing closestMark/currentSelectionNode helpers. No sanitizer change needed -- IMPORT_ALLOWED_TAGS already keeps MARK through the paste/upload sanitizer and through the split into sections, so a highlighted quote survives into whatever Prepare block it lands in.</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Verified with Playwright: selecting text in the Import stage and clicking the new button wraps it in &lt;mark&gt;; clicking again while selection sits inside an existing mark unwraps it; applying the staged content into a sermon carries the &lt;mark&gt; through into the resulting Prepare item's stored HTML intact. 6/6 checks passed, no page errors. Bumped sw.js v102-&gt;v103.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix native Google sign-in silently failing on trailing "#" in OAuth callback
Diagnosed live via Xcode console output: the appUrlOpen deep-link handler
was receiving the OAuth callback URL correctly (with the right PKCE code),
but sometimes with a bare trailing "#" and nothing after it. The
query-string parsing didn't strip that before handing the string to
URLSearchParams, which has no concept of "#" as a fragment delimiter --
the trailing "#" ended up glued onto the parsed code itself, and
exchangeCodeForSession silently rejected the corrupted value with no
error surfaced. Pre-existing bug, unrelated to the bundle-ID rename;
just hadn't been triggered/noticed before.

Ticket #91.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -627,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J94"/>
+  <dimension ref="A1:J95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5206,6 +5206,56 @@
       <c r="J94" t="inlineStr">
         <is>
           <t>Verified with a full git grep sweep across every tracked file (excluding context.md's history) confirming zero remaining com.shema.app references, a syntax check on index.html's script block, and a plist-parse check on the edited Info.plist. NOT yet verified: an actual Xcode build/run against the new identifier (needs the user's Mac). Two things only the user can do next: (1) add com.radahindustries.shema://auth-callback to Supabase Authentication &gt; URL Configuration &gt; Redirect URLs before native sign-in will work again; (2) on their Mac, git pull + npm install + npm run sync + re-run from Xcode. The original com.shema.app Apple-side limbo is left unresolved by choice -- reclaiming it later would need an Apple Developer Support ticket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>91</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Account/Auth</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Native Google sign-in silently fails: trailing "#" corrupts the PKCE code</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Right after getting the app building again on the new bundle ID, user reported Google sign-in completing the whole flow (Google auth, redirect back into the app) but landing back signed out, with no error message anywhere on screen.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Diagnosed live via Xcode console output while the user retried the flow with the device plugged in. The appUrlOpen deep-link event fires correctly with the right code -- captured URL: "com.radahindustries.shema://auth-callback?code=&lt;uuid&gt;#" -- confirming scheme registration, the Capacitor App plugin, and Supabase's redirect URL allow-list are all fine. The actual bug: the callback URL sometimes arrives with a bare trailing "#" (the marker itself, nothing after it), and the query-string parsing (url.split('?')[1]) does not strip that off before handing the string to URLSearchParams, which has no concept of "#" meaning "fragment starts here." The trailing "#" ends up glued onto the end of the last parsed value -- here, the PKCE code itself -- so exchangeCodeForSession silently gets a corrupted code and Supabase rejects it with no error surfaced back to the user. Pre-existing bug, unrelated to the same-day bundle-ID rename; it just had not been triggered/noticed before.</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Fixed by stripping anything from '#' onward out of the query-string half before parsing: const q = (url.split('?')[1] || '').split('#')[0];. Verified against the exact captured URL that this now extracts the clean UUID with no trailing character, and confirmed the fragment-based redirect branch (no '?' at all, e.g. ...auth-callback#access_token=...) is untouched by the change.</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Verified with a direct Node repro of the exact URL string, confirming the parsed code now matches the real UUID exactly. NOT yet verified against a real completed sign-in on the user's device -- next step is git pull + npm run sync + rebuild from Xcode, then retry Continue with Google. Bumped sw.js v105-&gt;v106.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Confirm native Google sign-in fixed end-to-end (ticket #91)
User confirmed a clean sign-in test succeeded on both iPhone and iPad:
exchange result {hasSession:true, error:null}, Account screen shows
signed in.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -5240,7 +5240,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Fixed by stripping anything from '#' onward out of the query-string half before parsing: const q = (url.split('?')[1] || '').split('#')[0];. Verified against the exact captured URL that this now extracts the clean UUID with no trailing character, and confirmed the fragment-based redirect branch (no '?' at all, e.g. ...auth-callback#access_token=...) is untouched by the change.</t>
+          <t>Fixed by stripping anything from '#' onward out of the query-string half before parsing: const q = (url.split('?')[1] || '').split('#')[0];. Verified against the exact captured URL that this now extracts the clean UUID with no trailing character, and confirmed the fragment-based redirect branch (no '?' at all, e.g. ...auth-callback#access_token=...) is untouched by the change. FOLLOW-UP FIXES: exchangeCodeForSession resolves to {data, error} rather than throwing -- the handler awaited it without checking .error, so a failed exchange had nothing to catch (no console.error, no toast). Added an explicit throw on a returned error, plus direct diagnostic console.log calls at handler entry, after parsing the code, and after the exchange call (logging hasSession + error) to remove all remaining guesswork. Left the diagnostic logs in place permanently -- cheap, useful breadcrumbs for next time, and they only fire during the native OAuth callback.</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -5250,12 +5250,12 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>Verified with a direct Node repro of the exact URL string, confirming the parsed code now matches the real UUID exactly. NOT yet verified against a real completed sign-in on the user's device -- next step is git pull + npm run sync + rebuild from Xcode, then retry Continue with Google. Bumped sw.js v105-&gt;v106.</t>
+          <t>Verified with a direct Node repro of the exact URL string, confirming the parsed code now matches the real UUID exactly. NOT yet verified against a real completed sign-in on the user's device -- next step is git pull + npm run sync + rebuild from Xcode, then retry Continue with Google. Bumped sw.js v105-&gt;v106. CONFIRMED WORKING 2026-09-03: user completed a clean single-tap sign-in test and the console showed exchange result {hasSession:true, error:null}; Account screen confirmed signed in. Verified on both iPhone and iPad. Bumped sw.js v106-&gt;v108 across the two follow-up commits.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix column mixup from previous tracker update (ticket #91 status/date)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -5245,12 +5245,12 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Needs Testing</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">

</xml_diff>

<commit_message>
Mark ticket #90 (bundle ID rename) Done -- confirmed working on-device
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -5195,7 +5195,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Needs Testing</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Verified with a full git grep sweep across every tracked file (excluding context.md's history) confirming zero remaining com.shema.app references, a syntax check on index.html's script block, and a plist-parse check on the edited Info.plist. NOT yet verified: an actual Xcode build/run against the new identifier (needs the user's Mac). Two things only the user can do next: (1) add com.radahindustries.shema://auth-callback to Supabase Authentication &gt; URL Configuration &gt; Redirect URLs before native sign-in will work again; (2) on their Mac, git pull + npm install + npm run sync + re-run from Xcode. The original com.shema.app Apple-side limbo is left unresolved by choice -- reclaiming it later would need an Apple Developer Support ticket.</t>
+          <t>Verified with a full git grep sweep across every tracked file (excluding context.md's history) confirming zero remaining com.shema.app references, a syntax check on index.html's script block, and a plist-parse check on the edited Info.plist. NOT yet verified: an actual Xcode build/run against the new identifier (needs the user's Mac). Two things only the user can do next: (1) add com.radahindustries.shema://auth-callback to Supabase Authentication &gt; URL Configuration &gt; Redirect URLs before native sign-in will work again; (2) on their Mac, git pull + npm install + npm run sync + re-run from Xcode. The original com.shema.app Apple-side limbo is left unresolved by choice -- reclaiming it later would need an Apple Developer Support ticket. CONFIRMED 2026-09-03: app builds and runs successfully on both iPhone and iPad under the new bundle ID, native Google sign-in also confirmed working end to end (see ticket #91).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log ticket #92 (&nbsp;/&amp; editor bug) and context.md entry
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -627,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5256,6 +5256,56 @@
       <c r="J95" t="inlineStr">
         <is>
           <t>Verified with a direct Node repro of the exact URL string, confirming the parsed code now matches the real UUID exactly. NOT yet verified against a real completed sign-in on the user's device -- next step is git pull + npm run sync + rebuild from Xcode, then retry Continue with Google. Bumped sw.js v105-&gt;v106. CONFIRMED WORKING 2026-09-03: user completed a clean single-tap sign-in test and the console showed exchange result {hasSession:true, error:null}; Account screen confirmed signed in. Verified on both iPhone and iPad. Bumped sw.js v106-&gt;v108 across the two follow-up commits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>92</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Prepare/Editor</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Fix &amp;nbsp;/&amp;amp; showing up as literal visible text in Prepare</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>User (dogfooding a real sermon in the app for the first time) spotted "&amp;nbsp;" appearing as literal on-screen text inside an item, live in the editor -- not in an exported file.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Same class of bug as #85's &amp;nbsp; leak in the ProPresenter export, but this time in the core editor render path #85 never touched. seedRichHtml and htmlToPlainText both decide legacy-plain-text vs. already-rich-HTML purely by checking for a '&lt;' character. A tag-free item (a bare '&amp;' or a non-breaking space typed/pasted with nothing else around it) gets correctly saved as real HTML the moment it's first edited -- the browser's own innerHTML serialization always round-trips a literal '&amp;' or NBSP as an entity, tag or no tag -- but that saved string then has zero '&lt;' characters in it. On the next render, both functions misread the entity-only string as legacy plain text and ran it through escapeHtml() a second time, turning a real '&amp;' into visible '&amp;amp;' or a real non-breaking space into visible '&amp;nbsp;' on screen. Not paste-specific: plain typing of an ampersand triggers it just as reliably on the next reload.</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Both functions now also accept a genuine HTML entity reference (&amp;amp;, &amp;nbsp;, &amp;#39;, ...) as equally valid proof a string is already real HTML, via a shared HTML_ENTITY_RE regex, alongside the existing '&lt;' check.</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Verified with a direct repro: a stored tag-free string containing &amp;nbsp; now passes through unchanged and renders as a real space; a genuinely bare legacy string ('Smith &amp; Sons') still correctly escapes on its first pass and is correctly recognized as already-HTML on every render after. This is prevention only -- any item already showing the literal text right now is already corrupted in storage from a prior render cycle and needs a one-time manual retype (delete the stray text, retype the space/ampersand); no auto-repair migration exists for already-corrupted text. Bumped sw.js v108-&gt;v109.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log ticket #93 (type-and-go click-to-add-line)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BrtijXUzSpiFaFhDEvEPsV
</commit_message>
<xml_diff>
--- a/Shema_Tickets.xlsx
+++ b/Shema_Tickets.xlsx
@@ -627,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5306,6 +5306,56 @@
       <c r="J96" t="inlineStr">
         <is>
           <t>Verified with a direct repro: a stored tag-free string containing &amp;nbsp; now passes through unchanged and renders as a real space; a genuinely bare legacy string ('Smith &amp; Sons') still correctly escapes on its first pass and is correctly recognized as already-HTML on every render after. This is prevention only -- any item already showing the literal text right now is already corrupted in storage from a prior render cycle and needs a one-time manual retype (delete the stray text, retype the space/ampersand); no auto-repair migration exists for already-corrupted text. Bumped sw.js v108-&gt;v109.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>93</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Prepare/Editor</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>"Type and go" click-to-add-line as an alternative to drag-a-chip</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>While writing a sermon on a laptop, user found the existing "+" popover drag-a-type-chip-onto-a-section mechanic (built with touch in mind) cumbersome with a mouse.</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Presented four alternatives with tradeoffs (per-section "+" dropdown, click-to-arm-then-click-target, always-visible icon row, editor-style type-and-go); user picked type-and-go. Added a plain-text click target at the end of every section's item list ("+ Add a line", or "Click to start writing..." when empty, replacing the old static empty-state message). Clicking it immediately creates a blank block item and focuses its text field -- click, then type, no menu. Switching the new item to scripture/quiet reuses the existing per-item type dropdown. Illustrations are intentionally excluded (pick-existing-content flow, not type-into-it) and still come from the "+" menu, which is otherwise untouched -- purely additive.</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Needs Testing</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Verified with Playwright: correct label on empty vs. non-empty sections; clicking creates exactly one new block item, defaults to type "block", focuses its text field; typing immediately after the click lands in the new item; an existing item in a non-empty section is preserved alongside the new one. 11/11 checks, no page errors. Bumped sw.js v109-&gt;v110.</t>
         </is>
       </c>
     </row>

</xml_diff>